<commit_message>
Redakcja: persony 71515 75446 76344 77093 60504 76342 60502 76463 76467
Zestawy z karta Piotra dostaja wylacznie persony, opis pusty. Persony celowo
nie powtarzaja tego, co karta juz niesie (cechy modelu, zl/element, porownania
w serii) — dokladaja werdykt rodzicielski i odbior na Bricksecie.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017crJHR6y9z5CNDcwqQ2UYg
</commit_message>
<xml_diff>
--- a/materialy/kolejka-redakcyjna.xlsx
+++ b/materialy/kolejka-redakcyjna.xlsx
@@ -4988,10 +4988,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G123" s="8" t="inlineStr"/>
+      <c r="G123" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H123" s="7" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -5588,10 +5592,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G139" s="8" t="inlineStr"/>
+      <c r="G139" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H139" s="7" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -5622,10 +5630,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G140" s="4" t="inlineStr"/>
+      <c r="G140" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H140" s="3" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -6332,10 +6344,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G159" s="8" t="inlineStr"/>
+      <c r="G159" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H159" s="7" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -6936,10 +6952,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G175" s="8" t="inlineStr"/>
+      <c r="G175" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H175" s="7" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -6970,10 +6990,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G176" s="4" t="inlineStr"/>
+      <c r="G176" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H176" s="3" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -8692,10 +8716,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G225" s="8" t="inlineStr"/>
+      <c r="G225" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H225" s="7" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -9094,10 +9122,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G236" s="4" t="inlineStr"/>
+      <c r="G236" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H236" s="3" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -9128,10 +9160,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G237" s="8" t="inlineStr"/>
+      <c r="G237" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H237" s="7" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -37191,7 +37227,7 @@
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>279</v>
+        <v>288</v>
       </c>
     </row>
     <row r="29">
@@ -37201,7 +37237,7 @@
         </is>
       </c>
       <c r="B29" s="11" t="n">
-        <v>174</v>
+        <v>165</v>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
Karty Piotra P07 (zakres 76-150): import 65 kart + 10 nadpisanych
Rejestr kart 513 -> 578. Dziesiec zestawow (42689 43025 60502 71514 71858
75423 75452 76463 76467 80119) mialo karty ze starszej paczki w formacie
2-5 akapitow; zastapione jednolita wersja P07 zgodnie z decyzja Marka przy
poprzedniej paczce. Importer przeszedl bez blokad i bez nierozwiazanych
placeholderow — poprawki szablonu z poprzedniego commita trzymaja.

sety.json: 65 wpisow dostalo karte, wiec nasz opis ustapil (pole wyczyszczone,
persony zostaja). Liczba wpisow bez zmian (456).

Statusy: gotowe 353, do person 165, do opisania 491, nasz opis 86.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017crJHR6y9z5CNDcwqQ2UYg
</commit_message>
<xml_diff>
--- a/materialy/kolejka-redakcyjna.xlsx
+++ b/materialy/kolejka-redakcyjna.xlsx
@@ -7327,7 +7327,11 @@
       <c r="E185" s="9" t="n">
         <v>439.99</v>
       </c>
-      <c r="F185" s="8" t="inlineStr"/>
+      <c r="F185" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G185" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -7335,7 +7339,7 @@
       </c>
       <c r="H185" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -7361,7 +7365,11 @@
       <c r="E186" s="5" t="n">
         <v>439.99</v>
       </c>
-      <c r="F186" s="4" t="inlineStr"/>
+      <c r="F186" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G186" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -7369,7 +7377,7 @@
       </c>
       <c r="H186" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -7395,7 +7403,11 @@
       <c r="E187" s="9" t="n">
         <v>439.99</v>
       </c>
-      <c r="F187" s="8" t="inlineStr"/>
+      <c r="F187" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G187" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -7403,7 +7415,7 @@
       </c>
       <c r="H187" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -7429,7 +7441,11 @@
       <c r="E188" s="5" t="n">
         <v>439.99</v>
       </c>
-      <c r="F188" s="4" t="inlineStr"/>
+      <c r="F188" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G188" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -7437,7 +7453,7 @@
       </c>
       <c r="H188" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -7463,7 +7479,11 @@
       <c r="E189" s="9" t="n">
         <v>439.99</v>
       </c>
-      <c r="F189" s="8" t="inlineStr"/>
+      <c r="F189" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G189" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -7471,7 +7491,7 @@
       </c>
       <c r="H189" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -7497,7 +7517,11 @@
       <c r="E190" s="5" t="n">
         <v>439.99</v>
       </c>
-      <c r="F190" s="4" t="inlineStr"/>
+      <c r="F190" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G190" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -7505,7 +7529,7 @@
       </c>
       <c r="H190" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -7531,7 +7555,11 @@
       <c r="E191" s="9" t="n">
         <v>439.99</v>
       </c>
-      <c r="F191" s="8" t="inlineStr"/>
+      <c r="F191" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G191" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -7539,7 +7567,7 @@
       </c>
       <c r="H191" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7593,11 @@
       <c r="E192" s="5" t="n">
         <v>429.99</v>
       </c>
-      <c r="F192" s="4" t="inlineStr"/>
+      <c r="F192" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G192" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -7573,7 +7605,7 @@
       </c>
       <c r="H192" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -7599,7 +7631,11 @@
       <c r="E193" s="9" t="n">
         <v>419.99</v>
       </c>
-      <c r="F193" s="8" t="inlineStr"/>
+      <c r="F193" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G193" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -7607,7 +7643,7 @@
       </c>
       <c r="H193" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -7633,7 +7669,11 @@
       <c r="E194" s="5" t="n">
         <v>419.99</v>
       </c>
-      <c r="F194" s="4" t="inlineStr"/>
+      <c r="F194" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G194" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -7641,7 +7681,7 @@
       </c>
       <c r="H194" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -7667,7 +7707,11 @@
       <c r="E195" s="9" t="n">
         <v>419.99</v>
       </c>
-      <c r="F195" s="8" t="inlineStr"/>
+      <c r="F195" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G195" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -7675,7 +7719,7 @@
       </c>
       <c r="H195" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -7701,7 +7745,11 @@
       <c r="E196" s="5" t="n">
         <v>419.99</v>
       </c>
-      <c r="F196" s="4" t="inlineStr"/>
+      <c r="F196" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G196" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -7709,7 +7757,7 @@
       </c>
       <c r="H196" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -7735,7 +7783,11 @@
       <c r="E197" s="9" t="n">
         <v>419.99</v>
       </c>
-      <c r="F197" s="8" t="inlineStr"/>
+      <c r="F197" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G197" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -7743,7 +7795,7 @@
       </c>
       <c r="H197" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -7769,7 +7821,11 @@
       <c r="E198" s="5" t="n">
         <v>419.99</v>
       </c>
-      <c r="F198" s="4" t="inlineStr"/>
+      <c r="F198" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G198" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -7777,7 +7833,7 @@
       </c>
       <c r="H198" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -7803,7 +7859,11 @@
       <c r="E199" s="9" t="n">
         <v>419.99</v>
       </c>
-      <c r="F199" s="8" t="inlineStr"/>
+      <c r="F199" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G199" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -7811,7 +7871,7 @@
       </c>
       <c r="H199" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7897,11 @@
       <c r="E200" s="5" t="n">
         <v>419.99</v>
       </c>
-      <c r="F200" s="4" t="inlineStr"/>
+      <c r="F200" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G200" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -7845,7 +7909,7 @@
       </c>
       <c r="H200" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -7871,7 +7935,11 @@
       <c r="E201" s="9" t="n">
         <v>419.99</v>
       </c>
-      <c r="F201" s="8" t="inlineStr"/>
+      <c r="F201" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G201" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -7879,7 +7947,7 @@
       </c>
       <c r="H201" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -7905,7 +7973,11 @@
       <c r="E202" s="5" t="n">
         <v>419.99</v>
       </c>
-      <c r="F202" s="4" t="inlineStr"/>
+      <c r="F202" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G202" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -7913,7 +7985,7 @@
       </c>
       <c r="H202" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -7939,7 +8011,11 @@
       <c r="E203" s="9" t="n">
         <v>419.99</v>
       </c>
-      <c r="F203" s="8" t="inlineStr"/>
+      <c r="F203" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G203" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -7947,7 +8023,7 @@
       </c>
       <c r="H203" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -7973,7 +8049,11 @@
       <c r="E204" s="5" t="n">
         <v>419.99</v>
       </c>
-      <c r="F204" s="4" t="inlineStr"/>
+      <c r="F204" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G204" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -7981,7 +8061,7 @@
       </c>
       <c r="H204" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -8007,7 +8087,11 @@
       <c r="E205" s="9" t="n">
         <v>419.99</v>
       </c>
-      <c r="F205" s="8" t="inlineStr"/>
+      <c r="F205" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G205" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -8015,7 +8099,7 @@
       </c>
       <c r="H205" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -8041,7 +8125,11 @@
       <c r="E206" s="5" t="n">
         <v>419.99</v>
       </c>
-      <c r="F206" s="4" t="inlineStr"/>
+      <c r="F206" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G206" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -8049,7 +8137,7 @@
       </c>
       <c r="H206" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -8075,7 +8163,11 @@
       <c r="E207" s="9" t="n">
         <v>419.99</v>
       </c>
-      <c r="F207" s="8" t="inlineStr"/>
+      <c r="F207" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G207" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -8083,7 +8175,7 @@
       </c>
       <c r="H207" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -8109,7 +8201,11 @@
       <c r="E208" s="5" t="n">
         <v>419.99</v>
       </c>
-      <c r="F208" s="4" t="inlineStr"/>
+      <c r="F208" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G208" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -8117,7 +8213,7 @@
       </c>
       <c r="H208" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -8143,7 +8239,11 @@
       <c r="E209" s="9" t="n">
         <v>419.99</v>
       </c>
-      <c r="F209" s="8" t="inlineStr"/>
+      <c r="F209" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G209" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -8151,7 +8251,7 @@
       </c>
       <c r="H209" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -8177,7 +8277,11 @@
       <c r="E210" s="5" t="n">
         <v>419.99</v>
       </c>
-      <c r="F210" s="4" t="inlineStr"/>
+      <c r="F210" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G210" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -8185,7 +8289,7 @@
       </c>
       <c r="H210" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -8211,7 +8315,11 @@
       <c r="E211" s="9" t="n">
         <v>419.99</v>
       </c>
-      <c r="F211" s="8" t="inlineStr"/>
+      <c r="F211" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G211" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -8219,7 +8327,7 @@
       </c>
       <c r="H211" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -8245,7 +8353,11 @@
       <c r="E212" s="5" t="n">
         <v>419.99</v>
       </c>
-      <c r="F212" s="4" t="inlineStr"/>
+      <c r="F212" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G212" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -8253,7 +8365,7 @@
       </c>
       <c r="H212" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -8279,7 +8391,11 @@
       <c r="E213" s="9" t="n">
         <v>419.99</v>
       </c>
-      <c r="F213" s="8" t="inlineStr"/>
+      <c r="F213" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G213" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -8287,7 +8403,7 @@
       </c>
       <c r="H213" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -8313,7 +8429,11 @@
       <c r="E214" s="5" t="n">
         <v>419.99</v>
       </c>
-      <c r="F214" s="4" t="inlineStr"/>
+      <c r="F214" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G214" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -8321,7 +8441,7 @@
       </c>
       <c r="H214" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -9417,7 +9537,11 @@
       <c r="E244" s="5" t="n">
         <v>409.99</v>
       </c>
-      <c r="F244" s="4" t="inlineStr"/>
+      <c r="F244" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G244" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -9425,7 +9549,7 @@
       </c>
       <c r="H244" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -9451,7 +9575,11 @@
       <c r="E245" s="9" t="n">
         <v>399.99</v>
       </c>
-      <c r="F245" s="8" t="inlineStr"/>
+      <c r="F245" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G245" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -9459,7 +9587,7 @@
       </c>
       <c r="H245" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -9485,7 +9613,11 @@
       <c r="E246" s="5" t="n">
         <v>399.99</v>
       </c>
-      <c r="F246" s="4" t="inlineStr"/>
+      <c r="F246" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G246" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -9493,7 +9625,7 @@
       </c>
       <c r="H246" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -9519,7 +9651,11 @@
       <c r="E247" s="9" t="n">
         <v>399.99</v>
       </c>
-      <c r="F247" s="8" t="inlineStr"/>
+      <c r="F247" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G247" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -9527,7 +9663,7 @@
       </c>
       <c r="H247" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -9553,7 +9689,11 @@
       <c r="E248" s="5" t="n">
         <v>389.99</v>
       </c>
-      <c r="F248" s="4" t="inlineStr"/>
+      <c r="F248" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G248" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -9561,7 +9701,7 @@
       </c>
       <c r="H248" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -9587,7 +9727,11 @@
       <c r="E249" s="9" t="n">
         <v>389.99</v>
       </c>
-      <c r="F249" s="8" t="inlineStr"/>
+      <c r="F249" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G249" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -9595,7 +9739,7 @@
       </c>
       <c r="H249" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -9621,7 +9765,11 @@
       <c r="E250" s="5" t="n">
         <v>389.99</v>
       </c>
-      <c r="F250" s="4" t="inlineStr"/>
+      <c r="F250" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G250" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -9629,7 +9777,7 @@
       </c>
       <c r="H250" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -9655,7 +9803,11 @@
       <c r="E251" s="9" t="n">
         <v>379.99</v>
       </c>
-      <c r="F251" s="8" t="inlineStr"/>
+      <c r="F251" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G251" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -9663,7 +9815,7 @@
       </c>
       <c r="H251" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -9689,7 +9841,11 @@
       <c r="E252" s="5" t="n">
         <v>379.99</v>
       </c>
-      <c r="F252" s="4" t="inlineStr"/>
+      <c r="F252" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G252" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -9697,7 +9853,7 @@
       </c>
       <c r="H252" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -9723,7 +9879,11 @@
       <c r="E253" s="9" t="n">
         <v>379.99</v>
       </c>
-      <c r="F253" s="8" t="inlineStr"/>
+      <c r="F253" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G253" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -9731,7 +9891,7 @@
       </c>
       <c r="H253" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -9757,7 +9917,11 @@
       <c r="E254" s="5" t="n">
         <v>379.99</v>
       </c>
-      <c r="F254" s="4" t="inlineStr"/>
+      <c r="F254" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G254" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -9765,7 +9929,7 @@
       </c>
       <c r="H254" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -9791,7 +9955,11 @@
       <c r="E255" s="9" t="n">
         <v>379.99</v>
       </c>
-      <c r="F255" s="8" t="inlineStr"/>
+      <c r="F255" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G255" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -9799,7 +9967,7 @@
       </c>
       <c r="H255" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -9825,7 +9993,11 @@
       <c r="E256" s="5" t="n">
         <v>379.99</v>
       </c>
-      <c r="F256" s="4" t="inlineStr"/>
+      <c r="F256" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G256" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -9833,7 +10005,7 @@
       </c>
       <c r="H256" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -9859,7 +10031,11 @@
       <c r="E257" s="9" t="n">
         <v>379.99</v>
       </c>
-      <c r="F257" s="8" t="inlineStr"/>
+      <c r="F257" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G257" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -9867,7 +10043,7 @@
       </c>
       <c r="H257" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -10477,7 +10653,11 @@
       <c r="E274" s="5" t="n">
         <v>369.99</v>
       </c>
-      <c r="F274" s="4" t="inlineStr"/>
+      <c r="F274" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G274" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -10485,7 +10665,7 @@
       </c>
       <c r="H274" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -10511,7 +10691,11 @@
       <c r="E275" s="9" t="n">
         <v>369.99</v>
       </c>
-      <c r="F275" s="8" t="inlineStr"/>
+      <c r="F275" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G275" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -10519,7 +10703,7 @@
       </c>
       <c r="H275" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -10545,7 +10729,11 @@
       <c r="E276" s="5" t="n">
         <v>359.99</v>
       </c>
-      <c r="F276" s="4" t="inlineStr"/>
+      <c r="F276" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G276" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -10553,7 +10741,7 @@
       </c>
       <c r="H276" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -10579,7 +10767,11 @@
       <c r="E277" s="9" t="n">
         <v>359.99</v>
       </c>
-      <c r="F277" s="8" t="inlineStr"/>
+      <c r="F277" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G277" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -10587,7 +10779,7 @@
       </c>
       <c r="H277" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -10613,7 +10805,11 @@
       <c r="E278" s="5" t="n">
         <v>359.99</v>
       </c>
-      <c r="F278" s="4" t="inlineStr"/>
+      <c r="F278" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G278" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -10621,7 +10817,7 @@
       </c>
       <c r="H278" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -10647,7 +10843,11 @@
       <c r="E279" s="9" t="n">
         <v>359.99</v>
       </c>
-      <c r="F279" s="8" t="inlineStr"/>
+      <c r="F279" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G279" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -10655,7 +10855,7 @@
       </c>
       <c r="H279" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -10681,7 +10881,11 @@
       <c r="E280" s="5" t="n">
         <v>349.99</v>
       </c>
-      <c r="F280" s="4" t="inlineStr"/>
+      <c r="F280" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G280" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -10689,7 +10893,7 @@
       </c>
       <c r="H280" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -10715,7 +10919,11 @@
       <c r="E281" s="9" t="n">
         <v>349.99</v>
       </c>
-      <c r="F281" s="8" t="inlineStr"/>
+      <c r="F281" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G281" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -10723,7 +10931,7 @@
       </c>
       <c r="H281" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -10749,7 +10957,11 @@
       <c r="E282" s="5" t="n">
         <v>349.99</v>
       </c>
-      <c r="F282" s="4" t="inlineStr"/>
+      <c r="F282" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G282" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -10757,7 +10969,7 @@
       </c>
       <c r="H282" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -10783,7 +10995,11 @@
       <c r="E283" s="9" t="n">
         <v>349.99</v>
       </c>
-      <c r="F283" s="8" t="inlineStr"/>
+      <c r="F283" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G283" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -10791,7 +11007,7 @@
       </c>
       <c r="H283" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -10817,7 +11033,11 @@
       <c r="E284" s="5" t="n">
         <v>349.99</v>
       </c>
-      <c r="F284" s="4" t="inlineStr"/>
+      <c r="F284" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G284" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -10825,7 +11045,7 @@
       </c>
       <c r="H284" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -10851,7 +11071,11 @@
       <c r="E285" s="9" t="n">
         <v>339.99</v>
       </c>
-      <c r="F285" s="8" t="inlineStr"/>
+      <c r="F285" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G285" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -10859,7 +11083,7 @@
       </c>
       <c r="H285" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -10885,7 +11109,11 @@
       <c r="E286" s="5" t="n">
         <v>339.99</v>
       </c>
-      <c r="F286" s="4" t="inlineStr"/>
+      <c r="F286" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G286" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -10893,7 +11121,7 @@
       </c>
       <c r="H286" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -10919,7 +11147,11 @@
       <c r="E287" s="9" t="n">
         <v>339.99</v>
       </c>
-      <c r="F287" s="8" t="inlineStr"/>
+      <c r="F287" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G287" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -10927,7 +11159,7 @@
       </c>
       <c r="H287" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -10953,7 +11185,11 @@
       <c r="E288" s="5" t="n">
         <v>339.99</v>
       </c>
-      <c r="F288" s="4" t="inlineStr"/>
+      <c r="F288" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G288" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -10961,7 +11197,7 @@
       </c>
       <c r="H288" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -10987,7 +11223,11 @@
       <c r="E289" s="9" t="n">
         <v>339.99</v>
       </c>
-      <c r="F289" s="8" t="inlineStr"/>
+      <c r="F289" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G289" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -10995,7 +11235,7 @@
       </c>
       <c r="H289" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -11021,7 +11261,11 @@
       <c r="E290" s="5" t="n">
         <v>339.99</v>
       </c>
-      <c r="F290" s="4" t="inlineStr"/>
+      <c r="F290" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G290" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -11029,7 +11273,7 @@
       </c>
       <c r="H290" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -11055,7 +11299,11 @@
       <c r="E291" s="9" t="n">
         <v>339.99</v>
       </c>
-      <c r="F291" s="8" t="inlineStr"/>
+      <c r="F291" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G291" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -11063,7 +11311,7 @@
       </c>
       <c r="H291" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -11089,7 +11337,11 @@
       <c r="E292" s="5" t="n">
         <v>339.99</v>
       </c>
-      <c r="F292" s="4" t="inlineStr"/>
+      <c r="F292" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G292" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -11097,7 +11349,7 @@
       </c>
       <c r="H292" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -11123,7 +11375,11 @@
       <c r="E293" s="9" t="n">
         <v>339.99</v>
       </c>
-      <c r="F293" s="8" t="inlineStr"/>
+      <c r="F293" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G293" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -11131,7 +11387,7 @@
       </c>
       <c r="H293" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -11157,7 +11413,11 @@
       <c r="E294" s="5" t="n">
         <v>339.99</v>
       </c>
-      <c r="F294" s="4" t="inlineStr"/>
+      <c r="F294" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G294" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -11165,7 +11425,7 @@
       </c>
       <c r="H294" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -37227,7 +37487,7 @@
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>288</v>
+        <v>353</v>
       </c>
     </row>
     <row r="29">
@@ -37247,7 +37507,7 @@
         </is>
       </c>
       <c r="B30" s="11" t="n">
-        <v>151</v>
+        <v>86</v>
       </c>
     </row>
     <row r="31">

</xml_diff>

<commit_message>
Redakcja: persony 80119 71858 71514 43025 75423 75452 42689 75425 75441 76470
75425 SMART Play Kantyna: Brickset klasyfikuje ja jako zestaw ZGODNY z SMART
Play, nie startowy — nie ma w niej klocka SMART (ma go 75423, ktorego karta
wprost pisze, ze "nie wymaga kupowania SMART Bricka z innego zestawu").
Bez modulu ze startera interakcja nie zadziala; z pudelka to nie wynika,
wiec ostrzezenie idzie na poczatek persony rodzica.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017crJHR6y9z5CNDcwqQ2UYg
</commit_message>
<xml_diff>
--- a/materialy/kolejka-redakcyjna.xlsx
+++ b/materialy/kolejka-redakcyjna.xlsx
@@ -8688,10 +8688,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G221" s="8" t="inlineStr"/>
+      <c r="G221" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H221" s="7" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -8912,10 +8916,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G227" s="8" t="inlineStr"/>
+      <c r="G227" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H227" s="7" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -8946,10 +8954,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G228" s="4" t="inlineStr"/>
+      <c r="G228" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H228" s="3" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -9508,10 +9520,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G243" s="8" t="inlineStr"/>
+      <c r="G243" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H243" s="7" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -10256,10 +10272,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G263" s="8" t="inlineStr"/>
+      <c r="G263" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H263" s="7" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -10552,10 +10572,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G271" s="8" t="inlineStr"/>
+      <c r="G271" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H271" s="7" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -10586,10 +10610,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G272" s="4" t="inlineStr"/>
+      <c r="G272" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H272" s="3" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -11922,10 +11950,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G308" s="4" t="inlineStr"/>
+      <c r="G308" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H308" s="3" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -11956,10 +11988,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G309" s="8" t="inlineStr"/>
+      <c r="G309" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H309" s="7" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -12028,10 +12064,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G311" s="8" t="inlineStr"/>
+      <c r="G311" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H311" s="7" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -37487,7 +37527,7 @@
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>353</v>
+        <v>363</v>
       </c>
     </row>
     <row r="29">
@@ -37497,7 +37537,7 @@
         </is>
       </c>
       <c r="B29" s="11" t="n">
-        <v>165</v>
+        <v>155</v>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
Karty Piotra P07 (zakres 151-225): import 53 kart + 22 nadpisane
Rejestr kart 578 -> 631. Dwadziescia dwie karty ze starszej paczki zastapione
jednolita wersja P07 (75421 i 75422 mialy dotad po jednym akapicie).

75425: nowa karta sama tlumaczy, ze zestaw nie zawiera SMART Bricka —
to samo ostrzezenie bylo dotad w personie rodzica, wiec persona przestaje je
powtarzac i przenosi ciezar na decyzje zakupowa (czy dop�ata za system SMART
ma sens bez startera). Ustalenie z poprzedniego commita bylo trafne.

sety.json: 10 wpisow dostalo karte, nasz opis wyczyszczony. Wpisow bez zmian.
Statusy: gotowe 373, do person 198, do opisania 448, nasz opis 76.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017crJHR6y9z5CNDcwqQ2UYg
</commit_message>
<xml_diff>
--- a/materialy/kolejka-redakcyjna.xlsx
+++ b/materialy/kolejka-redakcyjna.xlsx
@@ -11479,7 +11479,11 @@
       <c r="E295" s="9" t="n">
         <v>339.99</v>
       </c>
-      <c r="F295" s="8" t="inlineStr"/>
+      <c r="F295" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G295" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -11487,7 +11491,7 @@
       </c>
       <c r="H295" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -11513,7 +11517,11 @@
       <c r="E296" s="5" t="n">
         <v>339.99</v>
       </c>
-      <c r="F296" s="4" t="inlineStr"/>
+      <c r="F296" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G296" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -11521,7 +11529,7 @@
       </c>
       <c r="H296" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -12131,7 +12139,11 @@
       <c r="E313" s="9" t="n">
         <v>329.99</v>
       </c>
-      <c r="F313" s="8" t="inlineStr"/>
+      <c r="F313" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G313" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -12139,7 +12151,7 @@
       </c>
       <c r="H313" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -12165,7 +12177,11 @@
       <c r="E314" s="5" t="n">
         <v>329.99</v>
       </c>
-      <c r="F314" s="4" t="inlineStr"/>
+      <c r="F314" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G314" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -12173,7 +12189,7 @@
       </c>
       <c r="H314" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -12199,7 +12215,11 @@
       <c r="E315" s="9" t="n">
         <v>329.99</v>
       </c>
-      <c r="F315" s="8" t="inlineStr"/>
+      <c r="F315" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G315" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -12207,7 +12227,7 @@
       </c>
       <c r="H315" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -12233,7 +12253,11 @@
       <c r="E316" s="5" t="n">
         <v>329.99</v>
       </c>
-      <c r="F316" s="4" t="inlineStr"/>
+      <c r="F316" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G316" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -12241,7 +12265,7 @@
       </c>
       <c r="H316" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -12267,7 +12291,11 @@
       <c r="E317" s="9" t="n">
         <v>329.99</v>
       </c>
-      <c r="F317" s="8" t="inlineStr"/>
+      <c r="F317" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G317" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -12275,7 +12303,7 @@
       </c>
       <c r="H317" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -12301,7 +12329,11 @@
       <c r="E318" s="5" t="n">
         <v>329.99</v>
       </c>
-      <c r="F318" s="4" t="inlineStr"/>
+      <c r="F318" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G318" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -12309,7 +12341,7 @@
       </c>
       <c r="H318" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -12335,7 +12367,11 @@
       <c r="E319" s="9" t="n">
         <v>329.99</v>
       </c>
-      <c r="F319" s="8" t="inlineStr"/>
+      <c r="F319" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G319" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -12343,7 +12379,7 @@
       </c>
       <c r="H319" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -12369,7 +12405,11 @@
       <c r="E320" s="5" t="n">
         <v>319.99</v>
       </c>
-      <c r="F320" s="4" t="inlineStr"/>
+      <c r="F320" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G320" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -12377,7 +12417,7 @@
       </c>
       <c r="H320" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -12509,11 +12549,15 @@
       <c r="E324" s="5" t="n">
         <v>309.99</v>
       </c>
-      <c r="F324" s="4" t="inlineStr"/>
+      <c r="F324" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G324" s="4" t="inlineStr"/>
       <c r="H324" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -12539,11 +12583,15 @@
       <c r="E325" s="9" t="n">
         <v>309.99</v>
       </c>
-      <c r="F325" s="8" t="inlineStr"/>
+      <c r="F325" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G325" s="8" t="inlineStr"/>
       <c r="H325" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -12569,11 +12617,15 @@
       <c r="E326" s="5" t="n">
         <v>309.99</v>
       </c>
-      <c r="F326" s="4" t="inlineStr"/>
+      <c r="F326" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G326" s="4" t="inlineStr"/>
       <c r="H326" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -12599,11 +12651,15 @@
       <c r="E327" s="9" t="n">
         <v>300.99</v>
       </c>
-      <c r="F327" s="8" t="inlineStr"/>
+      <c r="F327" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G327" s="8" t="inlineStr"/>
       <c r="H327" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -12629,11 +12685,15 @@
       <c r="E328" s="5" t="n">
         <v>299.99</v>
       </c>
-      <c r="F328" s="4" t="inlineStr"/>
+      <c r="F328" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G328" s="4" t="inlineStr"/>
       <c r="H328" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -12659,11 +12719,15 @@
       <c r="E329" s="9" t="n">
         <v>299.99</v>
       </c>
-      <c r="F329" s="8" t="inlineStr"/>
+      <c r="F329" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G329" s="8" t="inlineStr"/>
       <c r="H329" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -12689,11 +12753,15 @@
       <c r="E330" s="5" t="n">
         <v>299.99</v>
       </c>
-      <c r="F330" s="4" t="inlineStr"/>
+      <c r="F330" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G330" s="4" t="inlineStr"/>
       <c r="H330" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -12719,11 +12787,15 @@
       <c r="E331" s="9" t="n">
         <v>299.99</v>
       </c>
-      <c r="F331" s="8" t="inlineStr"/>
+      <c r="F331" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G331" s="8" t="inlineStr"/>
       <c r="H331" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -12749,11 +12821,15 @@
       <c r="E332" s="5" t="n">
         <v>299.99</v>
       </c>
-      <c r="F332" s="4" t="inlineStr"/>
+      <c r="F332" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G332" s="4" t="inlineStr"/>
       <c r="H332" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -12813,11 +12889,15 @@
       <c r="E334" s="5" t="n">
         <v>299.99</v>
       </c>
-      <c r="F334" s="4" t="inlineStr"/>
+      <c r="F334" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G334" s="4" t="inlineStr"/>
       <c r="H334" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -12843,11 +12923,15 @@
       <c r="E335" s="9" t="n">
         <v>299.99</v>
       </c>
-      <c r="F335" s="8" t="inlineStr"/>
+      <c r="F335" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G335" s="8" t="inlineStr"/>
       <c r="H335" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -12873,11 +12957,15 @@
       <c r="E336" s="5" t="n">
         <v>299.99</v>
       </c>
-      <c r="F336" s="4" t="inlineStr"/>
+      <c r="F336" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G336" s="4" t="inlineStr"/>
       <c r="H336" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -12903,11 +12991,15 @@
       <c r="E337" s="9" t="n">
         <v>299.99</v>
       </c>
-      <c r="F337" s="8" t="inlineStr"/>
+      <c r="F337" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G337" s="8" t="inlineStr"/>
       <c r="H337" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -12933,11 +13025,15 @@
       <c r="E338" s="5" t="n">
         <v>299.99</v>
       </c>
-      <c r="F338" s="4" t="inlineStr"/>
+      <c r="F338" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G338" s="4" t="inlineStr"/>
       <c r="H338" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -12963,11 +13059,15 @@
       <c r="E339" s="9" t="n">
         <v>299.99</v>
       </c>
-      <c r="F339" s="8" t="inlineStr"/>
+      <c r="F339" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G339" s="8" t="inlineStr"/>
       <c r="H339" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -12993,11 +13093,15 @@
       <c r="E340" s="5" t="n">
         <v>299.99</v>
       </c>
-      <c r="F340" s="4" t="inlineStr"/>
+      <c r="F340" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G340" s="4" t="inlineStr"/>
       <c r="H340" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -13023,11 +13127,15 @@
       <c r="E341" s="9" t="n">
         <v>299.99</v>
       </c>
-      <c r="F341" s="8" t="inlineStr"/>
+      <c r="F341" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G341" s="8" t="inlineStr"/>
       <c r="H341" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -13053,11 +13161,15 @@
       <c r="E342" s="5" t="n">
         <v>299.99</v>
       </c>
-      <c r="F342" s="4" t="inlineStr"/>
+      <c r="F342" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G342" s="4" t="inlineStr"/>
       <c r="H342" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -13083,11 +13195,15 @@
       <c r="E343" s="9" t="n">
         <v>299.99</v>
       </c>
-      <c r="F343" s="8" t="inlineStr"/>
+      <c r="F343" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G343" s="8" t="inlineStr"/>
       <c r="H343" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -13113,11 +13229,15 @@
       <c r="E344" s="5" t="n">
         <v>299.99</v>
       </c>
-      <c r="F344" s="4" t="inlineStr"/>
+      <c r="F344" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G344" s="4" t="inlineStr"/>
       <c r="H344" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -13143,11 +13263,15 @@
       <c r="E345" s="9" t="n">
         <v>299.99</v>
       </c>
-      <c r="F345" s="8" t="inlineStr"/>
+      <c r="F345" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G345" s="8" t="inlineStr"/>
       <c r="H345" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -13173,11 +13297,15 @@
       <c r="E346" s="5" t="n">
         <v>299.99</v>
       </c>
-      <c r="F346" s="4" t="inlineStr"/>
+      <c r="F346" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G346" s="4" t="inlineStr"/>
       <c r="H346" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -13203,11 +13331,15 @@
       <c r="E347" s="9" t="n">
         <v>299.99</v>
       </c>
-      <c r="F347" s="8" t="inlineStr"/>
+      <c r="F347" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G347" s="8" t="inlineStr"/>
       <c r="H347" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -14101,11 +14233,15 @@
       <c r="E372" s="5" t="n">
         <v>289.99</v>
       </c>
-      <c r="F372" s="4" t="inlineStr"/>
+      <c r="F372" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G372" s="4" t="inlineStr"/>
       <c r="H372" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -14131,11 +14267,15 @@
       <c r="E373" s="9" t="n">
         <v>289.99</v>
       </c>
-      <c r="F373" s="8" t="inlineStr"/>
+      <c r="F373" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G373" s="8" t="inlineStr"/>
       <c r="H373" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -14161,11 +14301,15 @@
       <c r="E374" s="5" t="n">
         <v>279.99</v>
       </c>
-      <c r="F374" s="4" t="inlineStr"/>
+      <c r="F374" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G374" s="4" t="inlineStr"/>
       <c r="H374" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -14191,11 +14335,15 @@
       <c r="E375" s="9" t="n">
         <v>279.99</v>
       </c>
-      <c r="F375" s="8" t="inlineStr"/>
+      <c r="F375" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G375" s="8" t="inlineStr"/>
       <c r="H375" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -14221,11 +14369,15 @@
       <c r="E376" s="5" t="n">
         <v>279.99</v>
       </c>
-      <c r="F376" s="4" t="inlineStr"/>
+      <c r="F376" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G376" s="4" t="inlineStr"/>
       <c r="H376" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -14251,11 +14403,15 @@
       <c r="E377" s="9" t="n">
         <v>279.99</v>
       </c>
-      <c r="F377" s="8" t="inlineStr"/>
+      <c r="F377" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G377" s="8" t="inlineStr"/>
       <c r="H377" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -14281,11 +14437,15 @@
       <c r="E378" s="5" t="n">
         <v>279.99</v>
       </c>
-      <c r="F378" s="4" t="inlineStr"/>
+      <c r="F378" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G378" s="4" t="inlineStr"/>
       <c r="H378" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -14311,11 +14471,15 @@
       <c r="E379" s="9" t="n">
         <v>279.99</v>
       </c>
-      <c r="F379" s="8" t="inlineStr"/>
+      <c r="F379" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G379" s="8" t="inlineStr"/>
       <c r="H379" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -14341,11 +14505,15 @@
       <c r="E380" s="5" t="n">
         <v>274.99</v>
       </c>
-      <c r="F380" s="4" t="inlineStr"/>
+      <c r="F380" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G380" s="4" t="inlineStr"/>
       <c r="H380" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -14371,11 +14539,15 @@
       <c r="E381" s="9" t="n">
         <v>274.99</v>
       </c>
-      <c r="F381" s="8" t="inlineStr"/>
+      <c r="F381" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G381" s="8" t="inlineStr"/>
       <c r="H381" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -14401,11 +14573,15 @@
       <c r="E382" s="5" t="n">
         <v>274.99</v>
       </c>
-      <c r="F382" s="4" t="inlineStr"/>
+      <c r="F382" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G382" s="4" t="inlineStr"/>
       <c r="H382" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -14431,11 +14607,15 @@
       <c r="E383" s="9" t="n">
         <v>274.99</v>
       </c>
-      <c r="F383" s="8" t="inlineStr"/>
+      <c r="F383" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G383" s="8" t="inlineStr"/>
       <c r="H383" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -14461,11 +14641,15 @@
       <c r="E384" s="5" t="n">
         <v>274.99</v>
       </c>
-      <c r="F384" s="4" t="inlineStr"/>
+      <c r="F384" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G384" s="4" t="inlineStr"/>
       <c r="H384" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -14491,11 +14675,15 @@
       <c r="E385" s="9" t="n">
         <v>274.99</v>
       </c>
-      <c r="F385" s="8" t="inlineStr"/>
+      <c r="F385" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G385" s="8" t="inlineStr"/>
       <c r="H385" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -14881,11 +15069,15 @@
       <c r="E396" s="5" t="n">
         <v>269.99</v>
       </c>
-      <c r="F396" s="4" t="inlineStr"/>
+      <c r="F396" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G396" s="4" t="inlineStr"/>
       <c r="H396" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -14911,11 +15103,15 @@
       <c r="E397" s="9" t="n">
         <v>269.99</v>
       </c>
-      <c r="F397" s="8" t="inlineStr"/>
+      <c r="F397" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G397" s="8" t="inlineStr"/>
       <c r="H397" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -14941,11 +15137,15 @@
       <c r="E398" s="5" t="n">
         <v>269.99</v>
       </c>
-      <c r="F398" s="4" t="inlineStr"/>
+      <c r="F398" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G398" s="4" t="inlineStr"/>
       <c r="H398" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -14971,11 +15171,15 @@
       <c r="E399" s="9" t="n">
         <v>269.99</v>
       </c>
-      <c r="F399" s="8" t="inlineStr"/>
+      <c r="F399" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G399" s="8" t="inlineStr"/>
       <c r="H399" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -15001,11 +15205,15 @@
       <c r="E400" s="5" t="n">
         <v>259.99</v>
       </c>
-      <c r="F400" s="4" t="inlineStr"/>
+      <c r="F400" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G400" s="4" t="inlineStr"/>
       <c r="H400" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -15031,11 +15239,15 @@
       <c r="E401" s="9" t="n">
         <v>259.99</v>
       </c>
-      <c r="F401" s="8" t="inlineStr"/>
+      <c r="F401" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G401" s="8" t="inlineStr"/>
       <c r="H401" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -37517,7 +37729,7 @@
         </is>
       </c>
       <c r="B27" s="11" t="n">
-        <v>491</v>
+        <v>448</v>
       </c>
     </row>
     <row r="28">
@@ -37527,7 +37739,7 @@
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>363</v>
+        <v>373</v>
       </c>
     </row>
     <row r="29">
@@ -37537,7 +37749,7 @@
         </is>
       </c>
       <c r="B29" s="11" t="n">
-        <v>155</v>
+        <v>198</v>
       </c>
     </row>
     <row r="30">
@@ -37547,7 +37759,7 @@
         </is>
       </c>
       <c r="B30" s="11" t="n">
-        <v>86</v>
+        <v>76</v>
       </c>
     </row>
     <row r="31">

</xml_diff>

<commit_message>
Redakcja: persony 80118 42688 71857 71508 42223 75445 75328 76416 76433 42669
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017crJHR6y9z5CNDcwqQ2UYg
</commit_message>
<xml_diff>
--- a/materialy/kolejka-redakcyjna.xlsx
+++ b/materialy/kolejka-redakcyjna.xlsx
@@ -11746,10 +11746,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G302" s="4" t="inlineStr"/>
+      <c r="G302" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H302" s="3" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -11818,10 +11822,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G304" s="4" t="inlineStr"/>
+      <c r="G304" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H304" s="3" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -11852,10 +11860,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G305" s="8" t="inlineStr"/>
+      <c r="G305" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H305" s="7" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -12110,10 +12122,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G312" s="4" t="inlineStr"/>
+      <c r="G312" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H312" s="3" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -12486,10 +12502,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G322" s="4" t="inlineStr"/>
+      <c r="G322" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H322" s="3" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -12520,10 +12540,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G323" s="8" t="inlineStr"/>
+      <c r="G323" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H323" s="7" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -12554,10 +12578,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G324" s="4" t="inlineStr"/>
+      <c r="G324" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H324" s="3" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -12588,10 +12616,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G325" s="8" t="inlineStr"/>
+      <c r="G325" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H325" s="7" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -12622,10 +12654,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G326" s="4" t="inlineStr"/>
+      <c r="G326" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H326" s="3" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -12656,10 +12692,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G327" s="8" t="inlineStr"/>
+      <c r="G327" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H327" s="7" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -37739,7 +37779,7 @@
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>373</v>
+        <v>383</v>
       </c>
     </row>
     <row r="29">
@@ -37749,7 +37789,7 @@
         </is>
       </c>
       <c r="B29" s="11" t="n">
-        <v>198</v>
+        <v>188</v>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
Karty Piotra P07 (zakres 226-300): import 66 kart + 9 nadpisanych
Rejestr kart 631 -> 697. Import bez blokad. Zaden z dziewieciu nadpisanych
zestawow nie mial jeszcze naszej persony, wiec nie bylo ryzyka, ze nowa karta
zdubluje tekst persony.

Wszystkie 66 nowych kart trafilo na zestawy bez wpisu w sety.json, wiec nic
nie trzeba bylo czyscic; kolejka person rosnie do 254.

Statusy: gotowe 383, do person 254, do opisania 382, nasz opis 76.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017crJHR6y9z5CNDcwqQ2UYg
</commit_message>
<xml_diff>
--- a/materialy/kolejka-redakcyjna.xlsx
+++ b/materialy/kolejka-redakcyjna.xlsx
@@ -15313,11 +15313,15 @@
       <c r="E402" s="5" t="n">
         <v>259.99</v>
       </c>
-      <c r="F402" s="4" t="inlineStr"/>
+      <c r="F402" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G402" s="4" t="inlineStr"/>
       <c r="H402" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -15343,11 +15347,15 @@
       <c r="E403" s="9" t="n">
         <v>249.99</v>
       </c>
-      <c r="F403" s="8" t="inlineStr"/>
+      <c r="F403" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G403" s="8" t="inlineStr"/>
       <c r="H403" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -15373,11 +15381,15 @@
       <c r="E404" s="5" t="n">
         <v>249.99</v>
       </c>
-      <c r="F404" s="4" t="inlineStr"/>
+      <c r="F404" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G404" s="4" t="inlineStr"/>
       <c r="H404" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -15403,11 +15415,15 @@
       <c r="E405" s="9" t="n">
         <v>249.99</v>
       </c>
-      <c r="F405" s="8" t="inlineStr"/>
+      <c r="F405" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G405" s="8" t="inlineStr"/>
       <c r="H405" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -15433,11 +15449,15 @@
       <c r="E406" s="5" t="n">
         <v>249.99</v>
       </c>
-      <c r="F406" s="4" t="inlineStr"/>
+      <c r="F406" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G406" s="4" t="inlineStr"/>
       <c r="H406" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -15463,11 +15483,15 @@
       <c r="E407" s="9" t="n">
         <v>249.99</v>
       </c>
-      <c r="F407" s="8" t="inlineStr"/>
+      <c r="F407" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G407" s="8" t="inlineStr"/>
       <c r="H407" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -15493,11 +15517,15 @@
       <c r="E408" s="5" t="n">
         <v>249.99</v>
       </c>
-      <c r="F408" s="4" t="inlineStr"/>
+      <c r="F408" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G408" s="4" t="inlineStr"/>
       <c r="H408" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -15523,11 +15551,15 @@
       <c r="E409" s="9" t="n">
         <v>249.99</v>
       </c>
-      <c r="F409" s="8" t="inlineStr"/>
+      <c r="F409" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G409" s="8" t="inlineStr"/>
       <c r="H409" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -15553,11 +15585,15 @@
       <c r="E410" s="5" t="n">
         <v>249.99</v>
       </c>
-      <c r="F410" s="4" t="inlineStr"/>
+      <c r="F410" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G410" s="4" t="inlineStr"/>
       <c r="H410" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -15583,11 +15619,15 @@
       <c r="E411" s="9" t="n">
         <v>249.99</v>
       </c>
-      <c r="F411" s="8" t="inlineStr"/>
+      <c r="F411" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G411" s="8" t="inlineStr"/>
       <c r="H411" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -15613,11 +15653,15 @@
       <c r="E412" s="5" t="n">
         <v>249.99</v>
       </c>
-      <c r="F412" s="4" t="inlineStr"/>
+      <c r="F412" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G412" s="4" t="inlineStr"/>
       <c r="H412" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -15643,11 +15687,15 @@
       <c r="E413" s="9" t="n">
         <v>249.99</v>
       </c>
-      <c r="F413" s="8" t="inlineStr"/>
+      <c r="F413" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G413" s="8" t="inlineStr"/>
       <c r="H413" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -15673,11 +15721,15 @@
       <c r="E414" s="5" t="n">
         <v>249.99</v>
       </c>
-      <c r="F414" s="4" t="inlineStr"/>
+      <c r="F414" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G414" s="4" t="inlineStr"/>
       <c r="H414" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -15703,11 +15755,15 @@
       <c r="E415" s="9" t="n">
         <v>249.99</v>
       </c>
-      <c r="F415" s="8" t="inlineStr"/>
+      <c r="F415" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G415" s="8" t="inlineStr"/>
       <c r="H415" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -15733,11 +15789,15 @@
       <c r="E416" s="5" t="n">
         <v>249.99</v>
       </c>
-      <c r="F416" s="4" t="inlineStr"/>
+      <c r="F416" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G416" s="4" t="inlineStr"/>
       <c r="H416" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -15763,11 +15823,15 @@
       <c r="E417" s="9" t="n">
         <v>249.99</v>
       </c>
-      <c r="F417" s="8" t="inlineStr"/>
+      <c r="F417" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G417" s="8" t="inlineStr"/>
       <c r="H417" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -15793,11 +15857,15 @@
       <c r="E418" s="5" t="n">
         <v>249.99</v>
       </c>
-      <c r="F418" s="4" t="inlineStr"/>
+      <c r="F418" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G418" s="4" t="inlineStr"/>
       <c r="H418" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -15823,11 +15891,15 @@
       <c r="E419" s="9" t="n">
         <v>249.99</v>
       </c>
-      <c r="F419" s="8" t="inlineStr"/>
+      <c r="F419" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G419" s="8" t="inlineStr"/>
       <c r="H419" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -15853,11 +15925,15 @@
       <c r="E420" s="5" t="n">
         <v>249.99</v>
       </c>
-      <c r="F420" s="4" t="inlineStr"/>
+      <c r="F420" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G420" s="4" t="inlineStr"/>
       <c r="H420" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -15883,11 +15959,15 @@
       <c r="E421" s="9" t="n">
         <v>249.99</v>
       </c>
-      <c r="F421" s="8" t="inlineStr"/>
+      <c r="F421" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G421" s="8" t="inlineStr"/>
       <c r="H421" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -15913,11 +15993,15 @@
       <c r="E422" s="5" t="n">
         <v>249.99</v>
       </c>
-      <c r="F422" s="4" t="inlineStr"/>
+      <c r="F422" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G422" s="4" t="inlineStr"/>
       <c r="H422" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -15943,11 +16027,15 @@
       <c r="E423" s="9" t="n">
         <v>249.99</v>
       </c>
-      <c r="F423" s="8" t="inlineStr"/>
+      <c r="F423" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G423" s="8" t="inlineStr"/>
       <c r="H423" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -15973,11 +16061,15 @@
       <c r="E424" s="5" t="n">
         <v>249.99</v>
       </c>
-      <c r="F424" s="4" t="inlineStr"/>
+      <c r="F424" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G424" s="4" t="inlineStr"/>
       <c r="H424" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -16003,11 +16095,15 @@
       <c r="E425" s="9" t="n">
         <v>249.99</v>
       </c>
-      <c r="F425" s="8" t="inlineStr"/>
+      <c r="F425" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G425" s="8" t="inlineStr"/>
       <c r="H425" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -16033,11 +16129,15 @@
       <c r="E426" s="5" t="n">
         <v>249.99</v>
       </c>
-      <c r="F426" s="4" t="inlineStr"/>
+      <c r="F426" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G426" s="4" t="inlineStr"/>
       <c r="H426" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -16063,11 +16163,15 @@
       <c r="E427" s="9" t="n">
         <v>249.99</v>
       </c>
-      <c r="F427" s="8" t="inlineStr"/>
+      <c r="F427" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G427" s="8" t="inlineStr"/>
       <c r="H427" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -16237,11 +16341,15 @@
       <c r="E432" s="5" t="n">
         <v>249.99</v>
       </c>
-      <c r="F432" s="4" t="inlineStr"/>
+      <c r="F432" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G432" s="4" t="inlineStr"/>
       <c r="H432" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -16759,11 +16867,15 @@
       <c r="E447" s="9" t="n">
         <v>239.99</v>
       </c>
-      <c r="F447" s="8" t="inlineStr"/>
+      <c r="F447" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G447" s="8" t="inlineStr"/>
       <c r="H447" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -16789,11 +16901,15 @@
       <c r="E448" s="5" t="n">
         <v>239.99</v>
       </c>
-      <c r="F448" s="4" t="inlineStr"/>
+      <c r="F448" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G448" s="4" t="inlineStr"/>
       <c r="H448" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -16819,11 +16935,15 @@
       <c r="E449" s="9" t="n">
         <v>234.99</v>
       </c>
-      <c r="F449" s="8" t="inlineStr"/>
+      <c r="F449" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G449" s="8" t="inlineStr"/>
       <c r="H449" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -16849,11 +16969,15 @@
       <c r="E450" s="5" t="n">
         <v>234.99</v>
       </c>
-      <c r="F450" s="4" t="inlineStr"/>
+      <c r="F450" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G450" s="4" t="inlineStr"/>
       <c r="H450" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -16879,11 +17003,15 @@
       <c r="E451" s="9" t="n">
         <v>234.99</v>
       </c>
-      <c r="F451" s="8" t="inlineStr"/>
+      <c r="F451" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G451" s="8" t="inlineStr"/>
       <c r="H451" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -16909,11 +17037,15 @@
       <c r="E452" s="5" t="n">
         <v>234.99</v>
       </c>
-      <c r="F452" s="4" t="inlineStr"/>
+      <c r="F452" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G452" s="4" t="inlineStr"/>
       <c r="H452" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -16939,11 +17071,15 @@
       <c r="E453" s="9" t="n">
         <v>234.99</v>
       </c>
-      <c r="F453" s="8" t="inlineStr"/>
+      <c r="F453" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G453" s="8" t="inlineStr"/>
       <c r="H453" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -16969,11 +17105,15 @@
       <c r="E454" s="5" t="n">
         <v>234.99</v>
       </c>
-      <c r="F454" s="4" t="inlineStr"/>
+      <c r="F454" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G454" s="4" t="inlineStr"/>
       <c r="H454" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -16999,11 +17139,15 @@
       <c r="E455" s="9" t="n">
         <v>234.99</v>
       </c>
-      <c r="F455" s="8" t="inlineStr"/>
+      <c r="F455" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G455" s="8" t="inlineStr"/>
       <c r="H455" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17029,11 +17173,15 @@
       <c r="E456" s="5" t="n">
         <v>234.99</v>
       </c>
-      <c r="F456" s="4" t="inlineStr"/>
+      <c r="F456" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G456" s="4" t="inlineStr"/>
       <c r="H456" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17059,11 +17207,15 @@
       <c r="E457" s="9" t="n">
         <v>234.99</v>
       </c>
-      <c r="F457" s="8" t="inlineStr"/>
+      <c r="F457" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G457" s="8" t="inlineStr"/>
       <c r="H457" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17165,11 +17317,15 @@
       <c r="E460" s="5" t="n">
         <v>229.99</v>
       </c>
-      <c r="F460" s="4" t="inlineStr"/>
+      <c r="F460" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G460" s="4" t="inlineStr"/>
       <c r="H460" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17195,11 +17351,15 @@
       <c r="E461" s="9" t="n">
         <v>229.99</v>
       </c>
-      <c r="F461" s="8" t="inlineStr"/>
+      <c r="F461" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G461" s="8" t="inlineStr"/>
       <c r="H461" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17225,11 +17385,15 @@
       <c r="E462" s="5" t="n">
         <v>229.99</v>
       </c>
-      <c r="F462" s="4" t="inlineStr"/>
+      <c r="F462" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G462" s="4" t="inlineStr"/>
       <c r="H462" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17255,11 +17419,15 @@
       <c r="E463" s="9" t="n">
         <v>229.99</v>
       </c>
-      <c r="F463" s="8" t="inlineStr"/>
+      <c r="F463" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G463" s="8" t="inlineStr"/>
       <c r="H463" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17285,11 +17453,15 @@
       <c r="E464" s="5" t="n">
         <v>229.99</v>
       </c>
-      <c r="F464" s="4" t="inlineStr"/>
+      <c r="F464" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G464" s="4" t="inlineStr"/>
       <c r="H464" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17315,11 +17487,15 @@
       <c r="E465" s="9" t="n">
         <v>229.99</v>
       </c>
-      <c r="F465" s="8" t="inlineStr"/>
+      <c r="F465" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G465" s="8" t="inlineStr"/>
       <c r="H465" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17345,11 +17521,15 @@
       <c r="E466" s="5" t="n">
         <v>229.99</v>
       </c>
-      <c r="F466" s="4" t="inlineStr"/>
+      <c r="F466" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G466" s="4" t="inlineStr"/>
       <c r="H466" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17375,11 +17555,15 @@
       <c r="E467" s="9" t="n">
         <v>229.99</v>
       </c>
-      <c r="F467" s="8" t="inlineStr"/>
+      <c r="F467" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G467" s="8" t="inlineStr"/>
       <c r="H467" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17405,11 +17589,15 @@
       <c r="E468" s="5" t="n">
         <v>229.99</v>
       </c>
-      <c r="F468" s="4" t="inlineStr"/>
+      <c r="F468" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G468" s="4" t="inlineStr"/>
       <c r="H468" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17435,11 +17623,15 @@
       <c r="E469" s="9" t="n">
         <v>219.99</v>
       </c>
-      <c r="F469" s="8" t="inlineStr"/>
+      <c r="F469" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G469" s="8" t="inlineStr"/>
       <c r="H469" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17465,11 +17657,15 @@
       <c r="E470" s="5" t="n">
         <v>219.99</v>
       </c>
-      <c r="F470" s="4" t="inlineStr"/>
+      <c r="F470" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G470" s="4" t="inlineStr"/>
       <c r="H470" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17495,11 +17691,15 @@
       <c r="E471" s="9" t="n">
         <v>219.99</v>
       </c>
-      <c r="F471" s="8" t="inlineStr"/>
+      <c r="F471" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G471" s="8" t="inlineStr"/>
       <c r="H471" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17525,11 +17725,15 @@
       <c r="E472" s="5" t="n">
         <v>219.99</v>
       </c>
-      <c r="F472" s="4" t="inlineStr"/>
+      <c r="F472" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G472" s="4" t="inlineStr"/>
       <c r="H472" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17555,11 +17759,15 @@
       <c r="E473" s="9" t="n">
         <v>219.99</v>
       </c>
-      <c r="F473" s="8" t="inlineStr"/>
+      <c r="F473" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G473" s="8" t="inlineStr"/>
       <c r="H473" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17585,11 +17793,15 @@
       <c r="E474" s="5" t="n">
         <v>219.99</v>
       </c>
-      <c r="F474" s="4" t="inlineStr"/>
+      <c r="F474" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G474" s="4" t="inlineStr"/>
       <c r="H474" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17615,11 +17827,15 @@
       <c r="E475" s="9" t="n">
         <v>214.99</v>
       </c>
-      <c r="F475" s="8" t="inlineStr"/>
+      <c r="F475" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G475" s="8" t="inlineStr"/>
       <c r="H475" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17645,11 +17861,15 @@
       <c r="E476" s="5" t="n">
         <v>214.99</v>
       </c>
-      <c r="F476" s="4" t="inlineStr"/>
+      <c r="F476" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G476" s="4" t="inlineStr"/>
       <c r="H476" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17675,11 +17895,15 @@
       <c r="E477" s="9" t="n">
         <v>214.99</v>
       </c>
-      <c r="F477" s="8" t="inlineStr"/>
+      <c r="F477" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G477" s="8" t="inlineStr"/>
       <c r="H477" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17705,11 +17929,15 @@
       <c r="E478" s="5" t="n">
         <v>214.99</v>
       </c>
-      <c r="F478" s="4" t="inlineStr"/>
+      <c r="F478" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G478" s="4" t="inlineStr"/>
       <c r="H478" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17735,11 +17963,15 @@
       <c r="E479" s="9" t="n">
         <v>214.99</v>
       </c>
-      <c r="F479" s="8" t="inlineStr"/>
+      <c r="F479" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G479" s="8" t="inlineStr"/>
       <c r="H479" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17765,11 +17997,15 @@
       <c r="E480" s="5" t="n">
         <v>214.99</v>
       </c>
-      <c r="F480" s="4" t="inlineStr"/>
+      <c r="F480" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G480" s="4" t="inlineStr"/>
       <c r="H480" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17795,11 +18031,15 @@
       <c r="E481" s="9" t="n">
         <v>214.99</v>
       </c>
-      <c r="F481" s="8" t="inlineStr"/>
+      <c r="F481" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G481" s="8" t="inlineStr"/>
       <c r="H481" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17825,11 +18065,15 @@
       <c r="E482" s="5" t="n">
         <v>209.99</v>
       </c>
-      <c r="F482" s="4" t="inlineStr"/>
+      <c r="F482" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G482" s="4" t="inlineStr"/>
       <c r="H482" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17855,11 +18099,15 @@
       <c r="E483" s="9" t="n">
         <v>209.99</v>
       </c>
-      <c r="F483" s="8" t="inlineStr"/>
+      <c r="F483" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G483" s="8" t="inlineStr"/>
       <c r="H483" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17885,11 +18133,15 @@
       <c r="E484" s="5" t="n">
         <v>209.99</v>
       </c>
-      <c r="F484" s="4" t="inlineStr"/>
+      <c r="F484" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G484" s="4" t="inlineStr"/>
       <c r="H484" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17915,11 +18167,15 @@
       <c r="E485" s="9" t="n">
         <v>209.99</v>
       </c>
-      <c r="F485" s="8" t="inlineStr"/>
+      <c r="F485" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G485" s="8" t="inlineStr"/>
       <c r="H485" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17945,11 +18201,15 @@
       <c r="E486" s="5" t="n">
         <v>209.99</v>
       </c>
-      <c r="F486" s="4" t="inlineStr"/>
+      <c r="F486" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G486" s="4" t="inlineStr"/>
       <c r="H486" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -17975,11 +18235,15 @@
       <c r="E487" s="9" t="n">
         <v>209.99</v>
       </c>
-      <c r="F487" s="8" t="inlineStr"/>
+      <c r="F487" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G487" s="8" t="inlineStr"/>
       <c r="H487" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -37765,21 +38029,21 @@
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
       <c r="B27" s="11" t="n">
-        <v>448</v>
+        <v>383</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t>gotowe</t>
+          <t>do opisania</t>
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="29">
@@ -37789,7 +38053,7 @@
         </is>
       </c>
       <c r="B29" s="11" t="n">
-        <v>188</v>
+        <v>254</v>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
Redakcja: persony 60499 60505 75421 75422 75460 10467
Linia SMART Play: osiem zestawow na Bricksecie notuje oceny 2.9-4.1, tylko
jeden powyzej czworki, lacznie 74 glosy. Pojedynczo bazy sa za waskie na
wniosek, ale rozklad jest na tyle spojny, ze trafia do person 75421 i 75422
jako ostrzezenie przed wejsciem w caly system.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017crJHR6y9z5CNDcwqQ2UYg
</commit_message>
<xml_diff>
--- a/materialy/kolejka-redakcyjna.xlsx
+++ b/materialy/kolejka-redakcyjna.xlsx
@@ -13410,10 +13410,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G348" s="4" t="inlineStr"/>
+      <c r="G348" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H348" s="3" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -13668,10 +13672,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G355" s="8" t="inlineStr"/>
+      <c r="G355" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H355" s="7" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -13702,10 +13710,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G356" s="4" t="inlineStr"/>
+      <c r="G356" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H356" s="3" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -13948,10 +13960,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G363" s="8" t="inlineStr"/>
+      <c r="G363" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H363" s="7" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -13982,10 +13998,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G364" s="4" t="inlineStr"/>
+      <c r="G364" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H364" s="3" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -14054,10 +14074,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G366" s="4" t="inlineStr"/>
+      <c r="G366" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H366" s="3" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -38033,7 +38057,7 @@
         </is>
       </c>
       <c r="B27" s="11" t="n">
-        <v>383</v>
+        <v>389</v>
       </c>
     </row>
     <row r="28">
@@ -38053,7 +38077,7 @@
         </is>
       </c>
       <c r="B29" s="11" t="n">
-        <v>254</v>
+        <v>248</v>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
Karty Piotra P07 (zakres 301-375): import 54 kart + 21 nadpisanych
Rejestr kart 697 -> 751. Import bez blokad. Zaden z 21 nadpisanych zestawow
nie mial jeszcze persony, wiec kontrola pod katem dublowania wyszla pusta.

76924: Piotr podal 806 elementow, katalog i Brickset zgodnie 808 — metryka
karty bierze liczbe z repo, zeby nie przeczyla tabeli huba nad nia.

Statusy: gotowe 389, do person 302, do opisania 328, nasz opis 76.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017crJHR6y9z5CNDcwqQ2UYg
</commit_message>
<xml_diff>
--- a/materialy/kolejka-redakcyjna.xlsx
+++ b/materialy/kolejka-redakcyjna.xlsx
@@ -18293,11 +18293,15 @@
       <c r="E488" s="5" t="n">
         <v>209.99</v>
       </c>
-      <c r="F488" s="4" t="inlineStr"/>
+      <c r="F488" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G488" s="4" t="inlineStr"/>
       <c r="H488" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -18323,11 +18327,15 @@
       <c r="E489" s="9" t="n">
         <v>209.99</v>
       </c>
-      <c r="F489" s="8" t="inlineStr"/>
+      <c r="F489" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G489" s="8" t="inlineStr"/>
       <c r="H489" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -18353,11 +18361,15 @@
       <c r="E490" s="5" t="n">
         <v>209.99</v>
       </c>
-      <c r="F490" s="4" t="inlineStr"/>
+      <c r="F490" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G490" s="4" t="inlineStr"/>
       <c r="H490" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -18383,11 +18395,15 @@
       <c r="E491" s="9" t="n">
         <v>209.99</v>
       </c>
-      <c r="F491" s="8" t="inlineStr"/>
+      <c r="F491" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G491" s="8" t="inlineStr"/>
       <c r="H491" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -18413,11 +18429,15 @@
       <c r="E492" s="5" t="n">
         <v>209.99</v>
       </c>
-      <c r="F492" s="4" t="inlineStr"/>
+      <c r="F492" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G492" s="4" t="inlineStr"/>
       <c r="H492" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -18443,11 +18463,15 @@
       <c r="E493" s="9" t="n">
         <v>209.99</v>
       </c>
-      <c r="F493" s="8" t="inlineStr"/>
+      <c r="F493" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G493" s="8" t="inlineStr"/>
       <c r="H493" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -18473,11 +18497,15 @@
       <c r="E494" s="5" t="n">
         <v>209.99</v>
       </c>
-      <c r="F494" s="4" t="inlineStr"/>
+      <c r="F494" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G494" s="4" t="inlineStr"/>
       <c r="H494" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -18503,11 +18531,15 @@
       <c r="E495" s="9" t="n">
         <v>209.99</v>
       </c>
-      <c r="F495" s="8" t="inlineStr"/>
+      <c r="F495" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G495" s="8" t="inlineStr"/>
       <c r="H495" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -18533,11 +18565,15 @@
       <c r="E496" s="5" t="n">
         <v>209.99</v>
       </c>
-      <c r="F496" s="4" t="inlineStr"/>
+      <c r="F496" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G496" s="4" t="inlineStr"/>
       <c r="H496" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -18563,11 +18599,15 @@
       <c r="E497" s="9" t="n">
         <v>209.99</v>
       </c>
-      <c r="F497" s="8" t="inlineStr"/>
+      <c r="F497" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G497" s="8" t="inlineStr"/>
       <c r="H497" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -18593,11 +18633,15 @@
       <c r="E498" s="5" t="n">
         <v>209.99</v>
       </c>
-      <c r="F498" s="4" t="inlineStr"/>
+      <c r="F498" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G498" s="4" t="inlineStr"/>
       <c r="H498" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -18623,11 +18667,15 @@
       <c r="E499" s="9" t="n">
         <v>209.99</v>
       </c>
-      <c r="F499" s="8" t="inlineStr"/>
+      <c r="F499" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G499" s="8" t="inlineStr"/>
       <c r="H499" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -18653,11 +18701,15 @@
       <c r="E500" s="5" t="n">
         <v>209.99</v>
       </c>
-      <c r="F500" s="4" t="inlineStr"/>
+      <c r="F500" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G500" s="4" t="inlineStr"/>
       <c r="H500" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -18683,11 +18735,15 @@
       <c r="E501" s="9" t="n">
         <v>209.99</v>
       </c>
-      <c r="F501" s="8" t="inlineStr"/>
+      <c r="F501" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G501" s="8" t="inlineStr"/>
       <c r="H501" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -18713,11 +18769,15 @@
       <c r="E502" s="5" t="n">
         <v>209.99</v>
       </c>
-      <c r="F502" s="4" t="inlineStr"/>
+      <c r="F502" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G502" s="4" t="inlineStr"/>
       <c r="H502" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -18743,11 +18803,15 @@
       <c r="E503" s="9" t="n">
         <v>209.99</v>
       </c>
-      <c r="F503" s="8" t="inlineStr"/>
+      <c r="F503" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G503" s="8" t="inlineStr"/>
       <c r="H503" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -18773,11 +18837,15 @@
       <c r="E504" s="5" t="n">
         <v>209.99</v>
       </c>
-      <c r="F504" s="4" t="inlineStr"/>
+      <c r="F504" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G504" s="4" t="inlineStr"/>
       <c r="H504" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -18803,11 +18871,15 @@
       <c r="E505" s="9" t="n">
         <v>209.99</v>
       </c>
-      <c r="F505" s="8" t="inlineStr"/>
+      <c r="F505" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G505" s="8" t="inlineStr"/>
       <c r="H505" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -18833,11 +18905,15 @@
       <c r="E506" s="5" t="n">
         <v>209.99</v>
       </c>
-      <c r="F506" s="4" t="inlineStr"/>
+      <c r="F506" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G506" s="4" t="inlineStr"/>
       <c r="H506" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -18863,11 +18939,15 @@
       <c r="E507" s="9" t="n">
         <v>209.99</v>
       </c>
-      <c r="F507" s="8" t="inlineStr"/>
+      <c r="F507" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G507" s="8" t="inlineStr"/>
       <c r="H507" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -18893,11 +18973,15 @@
       <c r="E508" s="5" t="n">
         <v>209.99</v>
       </c>
-      <c r="F508" s="4" t="inlineStr"/>
+      <c r="F508" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G508" s="4" t="inlineStr"/>
       <c r="H508" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -19241,11 +19325,15 @@
       <c r="E518" s="5" t="n">
         <v>209.99</v>
       </c>
-      <c r="F518" s="4" t="inlineStr"/>
+      <c r="F518" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G518" s="4" t="inlineStr"/>
       <c r="H518" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -20241,11 +20329,15 @@
       <c r="E546" s="5" t="n">
         <v>199.99</v>
       </c>
-      <c r="F546" s="4" t="inlineStr"/>
+      <c r="F546" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G546" s="4" t="inlineStr"/>
       <c r="H546" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -20271,11 +20363,15 @@
       <c r="E547" s="9" t="n">
         <v>199.99</v>
       </c>
-      <c r="F547" s="8" t="inlineStr"/>
+      <c r="F547" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G547" s="8" t="inlineStr"/>
       <c r="H547" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -20301,11 +20397,15 @@
       <c r="E548" s="5" t="n">
         <v>199.99</v>
       </c>
-      <c r="F548" s="4" t="inlineStr"/>
+      <c r="F548" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G548" s="4" t="inlineStr"/>
       <c r="H548" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -20331,11 +20431,15 @@
       <c r="E549" s="9" t="n">
         <v>199.99</v>
       </c>
-      <c r="F549" s="8" t="inlineStr"/>
+      <c r="F549" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G549" s="8" t="inlineStr"/>
       <c r="H549" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -20361,11 +20465,15 @@
       <c r="E550" s="5" t="n">
         <v>189.99</v>
       </c>
-      <c r="F550" s="4" t="inlineStr"/>
+      <c r="F550" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G550" s="4" t="inlineStr"/>
       <c r="H550" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -20391,11 +20499,15 @@
       <c r="E551" s="9" t="n">
         <v>189.99</v>
       </c>
-      <c r="F551" s="8" t="inlineStr"/>
+      <c r="F551" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G551" s="8" t="inlineStr"/>
       <c r="H551" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -20421,11 +20533,15 @@
       <c r="E552" s="5" t="n">
         <v>189.99</v>
       </c>
-      <c r="F552" s="4" t="inlineStr"/>
+      <c r="F552" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G552" s="4" t="inlineStr"/>
       <c r="H552" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -20451,11 +20567,15 @@
       <c r="E553" s="9" t="n">
         <v>189.99</v>
       </c>
-      <c r="F553" s="8" t="inlineStr"/>
+      <c r="F553" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G553" s="8" t="inlineStr"/>
       <c r="H553" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -20481,11 +20601,15 @@
       <c r="E554" s="5" t="n">
         <v>189.99</v>
       </c>
-      <c r="F554" s="4" t="inlineStr"/>
+      <c r="F554" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G554" s="4" t="inlineStr"/>
       <c r="H554" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -20511,11 +20635,15 @@
       <c r="E555" s="9" t="n">
         <v>189.99</v>
       </c>
-      <c r="F555" s="8" t="inlineStr"/>
+      <c r="F555" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G555" s="8" t="inlineStr"/>
       <c r="H555" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -20541,11 +20669,15 @@
       <c r="E556" s="5" t="n">
         <v>189.99</v>
       </c>
-      <c r="F556" s="4" t="inlineStr"/>
+      <c r="F556" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G556" s="4" t="inlineStr"/>
       <c r="H556" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -20571,11 +20703,15 @@
       <c r="E557" s="9" t="n">
         <v>189.99</v>
       </c>
-      <c r="F557" s="8" t="inlineStr"/>
+      <c r="F557" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G557" s="8" t="inlineStr"/>
       <c r="H557" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -20601,11 +20737,15 @@
       <c r="E558" s="5" t="n">
         <v>189.99</v>
       </c>
-      <c r="F558" s="4" t="inlineStr"/>
+      <c r="F558" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G558" s="4" t="inlineStr"/>
       <c r="H558" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -20631,11 +20771,15 @@
       <c r="E559" s="9" t="n">
         <v>189.99</v>
       </c>
-      <c r="F559" s="8" t="inlineStr"/>
+      <c r="F559" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G559" s="8" t="inlineStr"/>
       <c r="H559" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -20661,11 +20805,15 @@
       <c r="E560" s="5" t="n">
         <v>189.99</v>
       </c>
-      <c r="F560" s="4" t="inlineStr"/>
+      <c r="F560" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G560" s="4" t="inlineStr"/>
       <c r="H560" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -20691,11 +20839,15 @@
       <c r="E561" s="9" t="n">
         <v>189.99</v>
       </c>
-      <c r="F561" s="8" t="inlineStr"/>
+      <c r="F561" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G561" s="8" t="inlineStr"/>
       <c r="H561" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -20721,11 +20873,15 @@
       <c r="E562" s="5" t="n">
         <v>189.99</v>
       </c>
-      <c r="F562" s="4" t="inlineStr"/>
+      <c r="F562" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G562" s="4" t="inlineStr"/>
       <c r="H562" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -20823,11 +20979,15 @@
       <c r="E565" s="9" t="n">
         <v>189.99</v>
       </c>
-      <c r="F565" s="8" t="inlineStr"/>
+      <c r="F565" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G565" s="8" t="inlineStr"/>
       <c r="H565" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -21027,11 +21187,15 @@
       <c r="E571" s="9" t="n">
         <v>184.99</v>
       </c>
-      <c r="F571" s="8" t="inlineStr"/>
+      <c r="F571" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G571" s="8" t="inlineStr"/>
       <c r="H571" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -21057,11 +21221,15 @@
       <c r="E572" s="5" t="n">
         <v>179.99</v>
       </c>
-      <c r="F572" s="4" t="inlineStr"/>
+      <c r="F572" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G572" s="4" t="inlineStr"/>
       <c r="H572" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -21087,11 +21255,15 @@
       <c r="E573" s="9" t="n">
         <v>179.99</v>
       </c>
-      <c r="F573" s="8" t="inlineStr"/>
+      <c r="F573" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G573" s="8" t="inlineStr"/>
       <c r="H573" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -21117,11 +21289,15 @@
       <c r="E574" s="5" t="n">
         <v>174.99</v>
       </c>
-      <c r="F574" s="4" t="inlineStr"/>
+      <c r="F574" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G574" s="4" t="inlineStr"/>
       <c r="H574" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -21147,11 +21323,15 @@
       <c r="E575" s="9" t="n">
         <v>174.99</v>
       </c>
-      <c r="F575" s="8" t="inlineStr"/>
+      <c r="F575" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G575" s="8" t="inlineStr"/>
       <c r="H575" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -21177,11 +21357,15 @@
       <c r="E576" s="5" t="n">
         <v>174.99</v>
       </c>
-      <c r="F576" s="4" t="inlineStr"/>
+      <c r="F576" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G576" s="4" t="inlineStr"/>
       <c r="H576" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -21207,11 +21391,15 @@
       <c r="E577" s="9" t="n">
         <v>174.99</v>
       </c>
-      <c r="F577" s="8" t="inlineStr"/>
+      <c r="F577" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G577" s="8" t="inlineStr"/>
       <c r="H577" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -21237,11 +21425,15 @@
       <c r="E578" s="5" t="n">
         <v>169.99</v>
       </c>
-      <c r="F578" s="4" t="inlineStr"/>
+      <c r="F578" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G578" s="4" t="inlineStr"/>
       <c r="H578" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -21267,11 +21459,15 @@
       <c r="E579" s="9" t="n">
         <v>169.99</v>
       </c>
-      <c r="F579" s="8" t="inlineStr"/>
+      <c r="F579" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G579" s="8" t="inlineStr"/>
       <c r="H579" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -21297,11 +21493,15 @@
       <c r="E580" s="5" t="n">
         <v>169.99</v>
       </c>
-      <c r="F580" s="4" t="inlineStr"/>
+      <c r="F580" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G580" s="4" t="inlineStr"/>
       <c r="H580" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -21327,11 +21527,15 @@
       <c r="E581" s="9" t="n">
         <v>169.99</v>
       </c>
-      <c r="F581" s="8" t="inlineStr"/>
+      <c r="F581" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G581" s="8" t="inlineStr"/>
       <c r="H581" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -21357,11 +21561,15 @@
       <c r="E582" s="5" t="n">
         <v>169.99</v>
       </c>
-      <c r="F582" s="4" t="inlineStr"/>
+      <c r="F582" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G582" s="4" t="inlineStr"/>
       <c r="H582" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -21387,11 +21595,15 @@
       <c r="E583" s="9" t="n">
         <v>169.99</v>
       </c>
-      <c r="F583" s="8" t="inlineStr"/>
+      <c r="F583" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G583" s="8" t="inlineStr"/>
       <c r="H583" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -21417,11 +21629,15 @@
       <c r="E584" s="5" t="n">
         <v>169.99</v>
       </c>
-      <c r="F584" s="4" t="inlineStr"/>
+      <c r="F584" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G584" s="4" t="inlineStr"/>
       <c r="H584" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -38067,7 +38283,7 @@
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>382</v>
+        <v>328</v>
       </c>
     </row>
     <row r="29">
@@ -38077,7 +38293,7 @@
         </is>
       </c>
       <c r="B29" s="11" t="n">
-        <v>248</v>
+        <v>302</v>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
Redakcja: persony 42687 10372 71512 10434 10451 10459
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017crJHR6y9z5CNDcwqQ2UYg
</commit_message>
<xml_diff>
--- a/materialy/kolejka-redakcyjna.xlsx
+++ b/materialy/kolejka-redakcyjna.xlsx
@@ -12798,10 +12798,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G330" s="4" t="inlineStr"/>
+      <c r="G330" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H330" s="3" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -12900,10 +12904,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G333" s="8" t="inlineStr"/>
+      <c r="G333" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H333" s="7" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -12934,10 +12942,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G334" s="4" t="inlineStr"/>
+      <c r="G334" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H334" s="3" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -12968,10 +12980,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G335" s="8" t="inlineStr"/>
+      <c r="G335" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H335" s="7" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -13524,10 +13540,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G351" s="8" t="inlineStr"/>
+      <c r="G351" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H351" s="7" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -13786,10 +13806,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G358" s="4" t="inlineStr"/>
+      <c r="G358" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H358" s="3" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -38273,7 +38297,7 @@
         </is>
       </c>
       <c r="B27" s="11" t="n">
-        <v>389</v>
+        <v>395</v>
       </c>
     </row>
     <row r="28">
@@ -38293,7 +38317,7 @@
         </is>
       </c>
       <c r="B29" s="11" t="n">
-        <v>302</v>
+        <v>296</v>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
Karty Piotra P07 (zakres 376-450): import 59 kart + 16 nadpisanych
Import bez blokad i bez rozbieznosci danych. Zaden z 16 nadpisanych zestawow
nie mial jeszcze persony, wiec kontrola pod katem dublowania wyszla pusta.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017crJHR6y9z5CNDcwqQ2UYg
</commit_message>
<xml_diff>
--- a/materialy/kolejka-redakcyjna.xlsx
+++ b/materialy/kolejka-redakcyjna.xlsx
@@ -21687,11 +21687,15 @@
       <c r="E585" s="9" t="n">
         <v>169.99</v>
       </c>
-      <c r="F585" s="8" t="inlineStr"/>
+      <c r="F585" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G585" s="8" t="inlineStr"/>
       <c r="H585" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -21717,11 +21721,15 @@
       <c r="E586" s="5" t="n">
         <v>169.99</v>
       </c>
-      <c r="F586" s="4" t="inlineStr"/>
+      <c r="F586" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G586" s="4" t="inlineStr"/>
       <c r="H586" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -21747,11 +21755,15 @@
       <c r="E587" s="9" t="n">
         <v>169.99</v>
       </c>
-      <c r="F587" s="8" t="inlineStr"/>
+      <c r="F587" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G587" s="8" t="inlineStr"/>
       <c r="H587" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -21777,11 +21789,15 @@
       <c r="E588" s="5" t="n">
         <v>169.99</v>
       </c>
-      <c r="F588" s="4" t="inlineStr"/>
+      <c r="F588" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G588" s="4" t="inlineStr"/>
       <c r="H588" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -21807,11 +21823,15 @@
       <c r="E589" s="9" t="n">
         <v>169.99</v>
       </c>
-      <c r="F589" s="8" t="inlineStr"/>
+      <c r="F589" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G589" s="8" t="inlineStr"/>
       <c r="H589" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -21837,11 +21857,15 @@
       <c r="E590" s="5" t="n">
         <v>169.99</v>
       </c>
-      <c r="F590" s="4" t="inlineStr"/>
+      <c r="F590" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G590" s="4" t="inlineStr"/>
       <c r="H590" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -21867,11 +21891,15 @@
       <c r="E591" s="9" t="n">
         <v>169.99</v>
       </c>
-      <c r="F591" s="8" t="inlineStr"/>
+      <c r="F591" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G591" s="8" t="inlineStr"/>
       <c r="H591" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -21897,11 +21925,15 @@
       <c r="E592" s="5" t="n">
         <v>169.99</v>
       </c>
-      <c r="F592" s="4" t="inlineStr"/>
+      <c r="F592" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G592" s="4" t="inlineStr"/>
       <c r="H592" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -21927,11 +21959,15 @@
       <c r="E593" s="9" t="n">
         <v>169.99</v>
       </c>
-      <c r="F593" s="8" t="inlineStr"/>
+      <c r="F593" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G593" s="8" t="inlineStr"/>
       <c r="H593" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -21957,11 +21993,15 @@
       <c r="E594" s="5" t="n">
         <v>169.99</v>
       </c>
-      <c r="F594" s="4" t="inlineStr"/>
+      <c r="F594" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G594" s="4" t="inlineStr"/>
       <c r="H594" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -21987,11 +22027,15 @@
       <c r="E595" s="9" t="n">
         <v>169.99</v>
       </c>
-      <c r="F595" s="8" t="inlineStr"/>
+      <c r="F595" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G595" s="8" t="inlineStr"/>
       <c r="H595" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -22017,11 +22061,15 @@
       <c r="E596" s="5" t="n">
         <v>169.99</v>
       </c>
-      <c r="F596" s="4" t="inlineStr"/>
+      <c r="F596" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G596" s="4" t="inlineStr"/>
       <c r="H596" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -22047,11 +22095,15 @@
       <c r="E597" s="9" t="n">
         <v>169.99</v>
       </c>
-      <c r="F597" s="8" t="inlineStr"/>
+      <c r="F597" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G597" s="8" t="inlineStr"/>
       <c r="H597" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -22077,11 +22129,15 @@
       <c r="E598" s="5" t="n">
         <v>169.99</v>
       </c>
-      <c r="F598" s="4" t="inlineStr"/>
+      <c r="F598" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G598" s="4" t="inlineStr"/>
       <c r="H598" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -22107,11 +22163,15 @@
       <c r="E599" s="9" t="n">
         <v>169.99</v>
       </c>
-      <c r="F599" s="8" t="inlineStr"/>
+      <c r="F599" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G599" s="8" t="inlineStr"/>
       <c r="H599" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -22137,11 +22197,15 @@
       <c r="E600" s="5" t="n">
         <v>169.99</v>
       </c>
-      <c r="F600" s="4" t="inlineStr"/>
+      <c r="F600" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G600" s="4" t="inlineStr"/>
       <c r="H600" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -22167,11 +22231,15 @@
       <c r="E601" s="9" t="n">
         <v>169.99</v>
       </c>
-      <c r="F601" s="8" t="inlineStr"/>
+      <c r="F601" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G601" s="8" t="inlineStr"/>
       <c r="H601" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -22197,11 +22265,15 @@
       <c r="E602" s="5" t="n">
         <v>169.99</v>
       </c>
-      <c r="F602" s="4" t="inlineStr"/>
+      <c r="F602" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G602" s="4" t="inlineStr"/>
       <c r="H602" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -22227,11 +22299,15 @@
       <c r="E603" s="9" t="n">
         <v>169.99</v>
       </c>
-      <c r="F603" s="8" t="inlineStr"/>
+      <c r="F603" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G603" s="8" t="inlineStr"/>
       <c r="H603" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -23223,11 +23299,15 @@
       <c r="E631" s="9" t="n">
         <v>159.99</v>
       </c>
-      <c r="F631" s="8" t="inlineStr"/>
+      <c r="F631" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G631" s="8" t="inlineStr"/>
       <c r="H631" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -23253,11 +23333,15 @@
       <c r="E632" s="5" t="n">
         <v>159.99</v>
       </c>
-      <c r="F632" s="4" t="inlineStr"/>
+      <c r="F632" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G632" s="4" t="inlineStr"/>
       <c r="H632" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -23283,11 +23367,15 @@
       <c r="E633" s="9" t="n">
         <v>159.99</v>
       </c>
-      <c r="F633" s="8" t="inlineStr"/>
+      <c r="F633" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G633" s="8" t="inlineStr"/>
       <c r="H633" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -23313,11 +23401,15 @@
       <c r="E634" s="5" t="n">
         <v>159.99</v>
       </c>
-      <c r="F634" s="4" t="inlineStr"/>
+      <c r="F634" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G634" s="4" t="inlineStr"/>
       <c r="H634" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -23343,11 +23435,15 @@
       <c r="E635" s="9" t="n">
         <v>159.99</v>
       </c>
-      <c r="F635" s="8" t="inlineStr"/>
+      <c r="F635" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G635" s="8" t="inlineStr"/>
       <c r="H635" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -23373,11 +23469,15 @@
       <c r="E636" s="5" t="n">
         <v>159.99</v>
       </c>
-      <c r="F636" s="4" t="inlineStr"/>
+      <c r="F636" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G636" s="4" t="inlineStr"/>
       <c r="H636" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -23403,11 +23503,15 @@
       <c r="E637" s="9" t="n">
         <v>149.99</v>
       </c>
-      <c r="F637" s="8" t="inlineStr"/>
+      <c r="F637" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G637" s="8" t="inlineStr"/>
       <c r="H637" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -23433,11 +23537,15 @@
       <c r="E638" s="5" t="n">
         <v>149.99</v>
       </c>
-      <c r="F638" s="4" t="inlineStr"/>
+      <c r="F638" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G638" s="4" t="inlineStr"/>
       <c r="H638" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -23463,11 +23571,15 @@
       <c r="E639" s="9" t="n">
         <v>149.99</v>
       </c>
-      <c r="F639" s="8" t="inlineStr"/>
+      <c r="F639" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G639" s="8" t="inlineStr"/>
       <c r="H639" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -23493,11 +23605,15 @@
       <c r="E640" s="5" t="n">
         <v>149.99</v>
       </c>
-      <c r="F640" s="4" t="inlineStr"/>
+      <c r="F640" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G640" s="4" t="inlineStr"/>
       <c r="H640" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -23523,11 +23639,15 @@
       <c r="E641" s="9" t="n">
         <v>149.99</v>
       </c>
-      <c r="F641" s="8" t="inlineStr"/>
+      <c r="F641" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G641" s="8" t="inlineStr"/>
       <c r="H641" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -23553,11 +23673,15 @@
       <c r="E642" s="5" t="n">
         <v>149.99</v>
       </c>
-      <c r="F642" s="4" t="inlineStr"/>
+      <c r="F642" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G642" s="4" t="inlineStr"/>
       <c r="H642" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -23583,11 +23707,15 @@
       <c r="E643" s="9" t="n">
         <v>149.99</v>
       </c>
-      <c r="F643" s="8" t="inlineStr"/>
+      <c r="F643" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G643" s="8" t="inlineStr"/>
       <c r="H643" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -23613,11 +23741,15 @@
       <c r="E644" s="5" t="n">
         <v>149.99</v>
       </c>
-      <c r="F644" s="4" t="inlineStr"/>
+      <c r="F644" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G644" s="4" t="inlineStr"/>
       <c r="H644" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -23643,11 +23775,15 @@
       <c r="E645" s="9" t="n">
         <v>149.99</v>
       </c>
-      <c r="F645" s="8" t="inlineStr"/>
+      <c r="F645" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G645" s="8" t="inlineStr"/>
       <c r="H645" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -23673,11 +23809,15 @@
       <c r="E646" s="5" t="n">
         <v>149.99</v>
       </c>
-      <c r="F646" s="4" t="inlineStr"/>
+      <c r="F646" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G646" s="4" t="inlineStr"/>
       <c r="H646" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -23703,11 +23843,15 @@
       <c r="E647" s="9" t="n">
         <v>149.99</v>
       </c>
-      <c r="F647" s="8" t="inlineStr"/>
+      <c r="F647" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G647" s="8" t="inlineStr"/>
       <c r="H647" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -23733,11 +23877,15 @@
       <c r="E648" s="5" t="n">
         <v>149.99</v>
       </c>
-      <c r="F648" s="4" t="inlineStr"/>
+      <c r="F648" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G648" s="4" t="inlineStr"/>
       <c r="H648" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -23763,11 +23911,15 @@
       <c r="E649" s="9" t="n">
         <v>144.99</v>
       </c>
-      <c r="F649" s="8" t="inlineStr"/>
+      <c r="F649" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G649" s="8" t="inlineStr"/>
       <c r="H649" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -23793,11 +23945,15 @@
       <c r="E650" s="5" t="n">
         <v>144.99</v>
       </c>
-      <c r="F650" s="4" t="inlineStr"/>
+      <c r="F650" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G650" s="4" t="inlineStr"/>
       <c r="H650" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -23823,11 +23979,15 @@
       <c r="E651" s="9" t="n">
         <v>144.99</v>
       </c>
-      <c r="F651" s="8" t="inlineStr"/>
+      <c r="F651" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G651" s="8" t="inlineStr"/>
       <c r="H651" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -23853,11 +24013,15 @@
       <c r="E652" s="5" t="n">
         <v>144.99</v>
       </c>
-      <c r="F652" s="4" t="inlineStr"/>
+      <c r="F652" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G652" s="4" t="inlineStr"/>
       <c r="H652" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -23883,11 +24047,15 @@
       <c r="E653" s="9" t="n">
         <v>144.99</v>
       </c>
-      <c r="F653" s="8" t="inlineStr"/>
+      <c r="F653" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G653" s="8" t="inlineStr"/>
       <c r="H653" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -23913,11 +24081,15 @@
       <c r="E654" s="5" t="n">
         <v>144.99</v>
       </c>
-      <c r="F654" s="4" t="inlineStr"/>
+      <c r="F654" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G654" s="4" t="inlineStr"/>
       <c r="H654" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -23943,11 +24115,15 @@
       <c r="E655" s="9" t="n">
         <v>144.99</v>
       </c>
-      <c r="F655" s="8" t="inlineStr"/>
+      <c r="F655" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G655" s="8" t="inlineStr"/>
       <c r="H655" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -24045,11 +24221,15 @@
       <c r="E658" s="5" t="n">
         <v>144.99</v>
       </c>
-      <c r="F658" s="4" t="inlineStr"/>
+      <c r="F658" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G658" s="4" t="inlineStr"/>
       <c r="H658" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -24075,11 +24255,15 @@
       <c r="E659" s="9" t="n">
         <v>144.99</v>
       </c>
-      <c r="F659" s="8" t="inlineStr"/>
+      <c r="F659" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G659" s="8" t="inlineStr"/>
       <c r="H659" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -24363,11 +24547,15 @@
       <c r="E667" s="9" t="n">
         <v>139.99</v>
       </c>
-      <c r="F667" s="8" t="inlineStr"/>
+      <c r="F667" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G667" s="8" t="inlineStr"/>
       <c r="H667" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -24393,11 +24581,15 @@
       <c r="E668" s="5" t="n">
         <v>139.99</v>
       </c>
-      <c r="F668" s="4" t="inlineStr"/>
+      <c r="F668" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G668" s="4" t="inlineStr"/>
       <c r="H668" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -24423,11 +24615,15 @@
       <c r="E669" s="9" t="n">
         <v>139.99</v>
       </c>
-      <c r="F669" s="8" t="inlineStr"/>
+      <c r="F669" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G669" s="8" t="inlineStr"/>
       <c r="H669" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -24453,11 +24649,15 @@
       <c r="E670" s="5" t="n">
         <v>129.99</v>
       </c>
-      <c r="F670" s="4" t="inlineStr"/>
+      <c r="F670" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G670" s="4" t="inlineStr"/>
       <c r="H670" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -24483,11 +24683,15 @@
       <c r="E671" s="9" t="n">
         <v>129.99</v>
       </c>
-      <c r="F671" s="8" t="inlineStr"/>
+      <c r="F671" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G671" s="8" t="inlineStr"/>
       <c r="H671" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -24513,11 +24717,15 @@
       <c r="E672" s="5" t="n">
         <v>129.99</v>
       </c>
-      <c r="F672" s="4" t="inlineStr"/>
+      <c r="F672" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G672" s="4" t="inlineStr"/>
       <c r="H672" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -24543,11 +24751,15 @@
       <c r="E673" s="9" t="n">
         <v>129.99</v>
       </c>
-      <c r="F673" s="8" t="inlineStr"/>
+      <c r="F673" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G673" s="8" t="inlineStr"/>
       <c r="H673" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -24573,11 +24785,15 @@
       <c r="E674" s="5" t="n">
         <v>129.99</v>
       </c>
-      <c r="F674" s="4" t="inlineStr"/>
+      <c r="F674" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G674" s="4" t="inlineStr"/>
       <c r="H674" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -24603,11 +24819,15 @@
       <c r="E675" s="9" t="n">
         <v>129.99</v>
       </c>
-      <c r="F675" s="8" t="inlineStr"/>
+      <c r="F675" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G675" s="8" t="inlineStr"/>
       <c r="H675" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -24633,11 +24853,15 @@
       <c r="E676" s="5" t="n">
         <v>129.99</v>
       </c>
-      <c r="F676" s="4" t="inlineStr"/>
+      <c r="F676" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G676" s="4" t="inlineStr"/>
       <c r="H676" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -24663,11 +24887,15 @@
       <c r="E677" s="9" t="n">
         <v>129.99</v>
       </c>
-      <c r="F677" s="8" t="inlineStr"/>
+      <c r="F677" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G677" s="8" t="inlineStr"/>
       <c r="H677" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -24693,11 +24921,15 @@
       <c r="E678" s="5" t="n">
         <v>129.99</v>
       </c>
-      <c r="F678" s="4" t="inlineStr"/>
+      <c r="F678" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G678" s="4" t="inlineStr"/>
       <c r="H678" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -24723,11 +24955,15 @@
       <c r="E679" s="9" t="n">
         <v>129.99</v>
       </c>
-      <c r="F679" s="8" t="inlineStr"/>
+      <c r="F679" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G679" s="8" t="inlineStr"/>
       <c r="H679" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -38303,21 +38539,21 @@
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>328</v>
+        <v>355</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>do opisania</t>
         </is>
       </c>
       <c r="B29" s="11" t="n">
-        <v>296</v>
+        <v>269</v>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
Redakcja: persony 21273 21357 42626 42652 42654 43240 43262 43279 71417 71843
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017crJHR6y9z5CNDcwqQ2UYg
</commit_message>
<xml_diff>
--- a/materialy/kolejka-redakcyjna.xlsx
+++ b/materialy/kolejka-redakcyjna.xlsx
@@ -12730,10 +12730,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G328" s="4" t="inlineStr"/>
+      <c r="G328" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H328" s="3" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -12836,10 +12840,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G331" s="8" t="inlineStr"/>
+      <c r="G331" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H331" s="7" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -12870,10 +12878,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G332" s="4" t="inlineStr"/>
+      <c r="G332" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H332" s="3" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -13018,10 +13030,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G336" s="4" t="inlineStr"/>
+      <c r="G336" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H336" s="3" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -13052,10 +13068,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G337" s="8" t="inlineStr"/>
+      <c r="G337" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H337" s="7" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -13086,10 +13106,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G338" s="4" t="inlineStr"/>
+      <c r="G338" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H338" s="3" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -13120,10 +13144,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G339" s="8" t="inlineStr"/>
+      <c r="G339" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H339" s="7" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -13154,10 +13182,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G340" s="4" t="inlineStr"/>
+      <c r="G340" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H340" s="3" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -13188,10 +13220,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G341" s="8" t="inlineStr"/>
+      <c r="G341" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H341" s="7" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -13222,10 +13258,14 @@
           <t>tak</t>
         </is>
       </c>
-      <c r="G342" s="4" t="inlineStr"/>
+      <c r="G342" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H342" s="3" t="inlineStr">
         <is>
-          <t>do person</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -38533,7 +38573,7 @@
         </is>
       </c>
       <c r="B27" s="11" t="n">
-        <v>395</v>
+        <v>405</v>
       </c>
     </row>
     <row r="28">
@@ -38543,7 +38583,7 @@
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>355</v>
+        <v>345</v>
       </c>
     </row>
     <row r="29">

</xml_diff>

<commit_message>
Karty Piotra P07 (zakres 451-480 + czesc paczki potwierdzonych): import 36 kart
Rejestr kart 810 -> 846. Kolejka 451-480 weszla bez zastrzezen (30 kart).
Z paczki "15 potwierdzonych zestawow 2026/2027" weszlo 6; 9 zostalo
wstrzymanych do decyzji Marka:
  - 8 zestawow nowej linii Super Mario 2027 (72052 72054-72058 72061)
    ma po jednym akapicie opisu i NIE ma rekordu w katalog.json, wiec ich
    karty nie mialyby gdzie sie wyswietlic;
  - 40862 i 40866 maja strony, ale rowniez po jednym akapicie, wiec zatrzymuje
    je zabezpieczenie wymagajace minimum dwoch.
Pliki parsuja sie poprawnie (metryka 12 pol, FAQ 6 pytan) — to nie jest blad
struktury, tylko krotsza karta.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017crJHR6y9z5CNDcwqQ2UYg
</commit_message>
<xml_diff>
--- a/materialy/kolejka-redakcyjna.xlsx
+++ b/materialy/kolejka-redakcyjna.xlsx
@@ -8467,7 +8467,11 @@
       <c r="E215" s="9" t="n">
         <v>419.99</v>
       </c>
-      <c r="F215" s="8" t="inlineStr"/>
+      <c r="F215" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G215" s="8" t="inlineStr">
         <is>
           <t>tak</t>
@@ -8475,7 +8479,7 @@
       </c>
       <c r="H215" s="7" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -16497,7 +16501,11 @@
       <c r="E434" s="5" t="n">
         <v>249.99</v>
       </c>
-      <c r="F434" s="4" t="inlineStr"/>
+      <c r="F434" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G434" s="4" t="inlineStr">
         <is>
           <t>tak</t>
@@ -16505,7 +16513,7 @@
       </c>
       <c r="H434" s="3" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -25029,11 +25037,15 @@
       <c r="E680" s="5" t="n">
         <v>129.99</v>
       </c>
-      <c r="F680" s="4" t="inlineStr"/>
+      <c r="F680" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G680" s="4" t="inlineStr"/>
       <c r="H680" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25059,11 +25071,15 @@
       <c r="E681" s="9" t="n">
         <v>129.99</v>
       </c>
-      <c r="F681" s="8" t="inlineStr"/>
+      <c r="F681" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G681" s="8" t="inlineStr"/>
       <c r="H681" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25089,11 +25105,15 @@
       <c r="E682" s="5" t="n">
         <v>129.99</v>
       </c>
-      <c r="F682" s="4" t="inlineStr"/>
+      <c r="F682" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G682" s="4" t="inlineStr"/>
       <c r="H682" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25119,11 +25139,15 @@
       <c r="E683" s="9" t="n">
         <v>129.99</v>
       </c>
-      <c r="F683" s="8" t="inlineStr"/>
+      <c r="F683" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G683" s="8" t="inlineStr"/>
       <c r="H683" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25149,11 +25173,15 @@
       <c r="E684" s="5" t="n">
         <v>124.99</v>
       </c>
-      <c r="F684" s="4" t="inlineStr"/>
+      <c r="F684" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G684" s="4" t="inlineStr"/>
       <c r="H684" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25179,11 +25207,15 @@
       <c r="E685" s="9" t="n">
         <v>124.99</v>
       </c>
-      <c r="F685" s="8" t="inlineStr"/>
+      <c r="F685" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G685" s="8" t="inlineStr"/>
       <c r="H685" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25209,11 +25241,15 @@
       <c r="E686" s="5" t="n">
         <v>124.99</v>
       </c>
-      <c r="F686" s="4" t="inlineStr"/>
+      <c r="F686" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G686" s="4" t="inlineStr"/>
       <c r="H686" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25239,11 +25275,15 @@
       <c r="E687" s="9" t="n">
         <v>124.99</v>
       </c>
-      <c r="F687" s="8" t="inlineStr"/>
+      <c r="F687" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G687" s="8" t="inlineStr"/>
       <c r="H687" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25269,11 +25309,15 @@
       <c r="E688" s="5" t="n">
         <v>124.99</v>
       </c>
-      <c r="F688" s="4" t="inlineStr"/>
+      <c r="F688" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G688" s="4" t="inlineStr"/>
       <c r="H688" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25299,11 +25343,15 @@
       <c r="E689" s="9" t="n">
         <v>124.99</v>
       </c>
-      <c r="F689" s="8" t="inlineStr"/>
+      <c r="F689" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G689" s="8" t="inlineStr"/>
       <c r="H689" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25329,11 +25377,15 @@
       <c r="E690" s="5" t="n">
         <v>124.99</v>
       </c>
-      <c r="F690" s="4" t="inlineStr"/>
+      <c r="F690" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G690" s="4" t="inlineStr"/>
       <c r="H690" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25359,11 +25411,15 @@
       <c r="E691" s="9" t="n">
         <v>124.99</v>
       </c>
-      <c r="F691" s="8" t="inlineStr"/>
+      <c r="F691" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G691" s="8" t="inlineStr"/>
       <c r="H691" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25389,11 +25445,15 @@
       <c r="E692" s="5" t="n">
         <v>124.99</v>
       </c>
-      <c r="F692" s="4" t="inlineStr"/>
+      <c r="F692" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G692" s="4" t="inlineStr"/>
       <c r="H692" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25419,11 +25479,15 @@
       <c r="E693" s="9" t="n">
         <v>124.99</v>
       </c>
-      <c r="F693" s="8" t="inlineStr"/>
+      <c r="F693" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G693" s="8" t="inlineStr"/>
       <c r="H693" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25449,11 +25513,15 @@
       <c r="E694" s="5" t="n">
         <v>124.99</v>
       </c>
-      <c r="F694" s="4" t="inlineStr"/>
+      <c r="F694" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G694" s="4" t="inlineStr"/>
       <c r="H694" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25479,11 +25547,15 @@
       <c r="E695" s="9" t="n">
         <v>124.99</v>
       </c>
-      <c r="F695" s="8" t="inlineStr"/>
+      <c r="F695" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G695" s="8" t="inlineStr"/>
       <c r="H695" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25509,11 +25581,15 @@
       <c r="E696" s="5" t="n">
         <v>124.99</v>
       </c>
-      <c r="F696" s="4" t="inlineStr"/>
+      <c r="F696" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G696" s="4" t="inlineStr"/>
       <c r="H696" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25539,11 +25615,15 @@
       <c r="E697" s="9" t="n">
         <v>124.99</v>
       </c>
-      <c r="F697" s="8" t="inlineStr"/>
+      <c r="F697" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G697" s="8" t="inlineStr"/>
       <c r="H697" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25569,11 +25649,15 @@
       <c r="E698" s="5" t="n">
         <v>124.99</v>
       </c>
-      <c r="F698" s="4" t="inlineStr"/>
+      <c r="F698" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G698" s="4" t="inlineStr"/>
       <c r="H698" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25599,11 +25683,15 @@
       <c r="E699" s="9" t="n">
         <v>124.99</v>
       </c>
-      <c r="F699" s="8" t="inlineStr"/>
+      <c r="F699" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G699" s="8" t="inlineStr"/>
       <c r="H699" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25629,11 +25717,15 @@
       <c r="E700" s="5" t="n">
         <v>124.99</v>
       </c>
-      <c r="F700" s="4" t="inlineStr"/>
+      <c r="F700" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G700" s="4" t="inlineStr"/>
       <c r="H700" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25659,11 +25751,15 @@
       <c r="E701" s="9" t="n">
         <v>124.99</v>
       </c>
-      <c r="F701" s="8" t="inlineStr"/>
+      <c r="F701" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G701" s="8" t="inlineStr"/>
       <c r="H701" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25689,11 +25785,15 @@
       <c r="E702" s="5" t="n">
         <v>124.99</v>
       </c>
-      <c r="F702" s="4" t="inlineStr"/>
+      <c r="F702" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G702" s="4" t="inlineStr"/>
       <c r="H702" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25719,11 +25819,15 @@
       <c r="E703" s="9" t="n">
         <v>124.99</v>
       </c>
-      <c r="F703" s="8" t="inlineStr"/>
+      <c r="F703" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G703" s="8" t="inlineStr"/>
       <c r="H703" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25749,11 +25853,15 @@
       <c r="E704" s="5" t="n">
         <v>124.99</v>
       </c>
-      <c r="F704" s="4" t="inlineStr"/>
+      <c r="F704" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G704" s="4" t="inlineStr"/>
       <c r="H704" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25779,11 +25887,15 @@
       <c r="E705" s="9" t="n">
         <v>124.99</v>
       </c>
-      <c r="F705" s="8" t="inlineStr"/>
+      <c r="F705" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G705" s="8" t="inlineStr"/>
       <c r="H705" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25809,11 +25921,15 @@
       <c r="E706" s="5" t="n">
         <v>124.99</v>
       </c>
-      <c r="F706" s="4" t="inlineStr"/>
+      <c r="F706" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G706" s="4" t="inlineStr"/>
       <c r="H706" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25839,11 +25955,15 @@
       <c r="E707" s="9" t="n">
         <v>124.99</v>
       </c>
-      <c r="F707" s="8" t="inlineStr"/>
+      <c r="F707" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G707" s="8" t="inlineStr"/>
       <c r="H707" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25869,11 +25989,15 @@
       <c r="E708" s="5" t="n">
         <v>124.99</v>
       </c>
-      <c r="F708" s="4" t="inlineStr"/>
+      <c r="F708" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G708" s="4" t="inlineStr"/>
       <c r="H708" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -25899,11 +26023,15 @@
       <c r="E709" s="9" t="n">
         <v>124.99</v>
       </c>
-      <c r="F709" s="8" t="inlineStr"/>
+      <c r="F709" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="G709" s="8" t="inlineStr"/>
       <c r="H709" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>do person</t>
         </is>
       </c>
     </row>
@@ -38573,7 +38701,7 @@
         </is>
       </c>
       <c r="B27" s="11" t="n">
-        <v>405</v>
+        <v>407</v>
       </c>
     </row>
     <row r="28">
@@ -38583,7 +38711,7 @@
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>345</v>
+        <v>375</v>
       </c>
     </row>
     <row r="29">
@@ -38593,7 +38721,7 @@
         </is>
       </c>
       <c r="B29" s="11" t="n">
-        <v>269</v>
+        <v>239</v>
       </c>
     </row>
     <row r="30">
@@ -38603,7 +38731,7 @@
         </is>
       </c>
       <c r="B30" s="11" t="n">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="31">

</xml_diff>

<commit_message>
Redakcja: 75 nowych kart Piotra i persony do wszystkich
- import 90 dokumentow: 75 nowych kart, 15 nadpisanych pelniejszymi wersjami
- persony (dla_rodzica + dla_afol) do wszystkich 75 zestawow: sety.json 935 -> 1010
- odswiezone listingi: kolejka redakcyjna, karty poza kolejka, zestawy bez ceny

Kolejka: gotowe 885 (bylo 810), do person 0, do opisania 164.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017crJHR6y9z5CNDcwqQ2UYg
</commit_message>
<xml_diff>
--- a/materialy/kolejka-redakcyjna.xlsx
+++ b/materialy/kolejka-redakcyjna.xlsx
@@ -27729,11 +27729,19 @@
       <c r="E724" s="5" t="n">
         <v>124.99</v>
       </c>
-      <c r="F724" s="4" t="inlineStr"/>
-      <c r="G724" s="4" t="inlineStr"/>
+      <c r="F724" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G724" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H724" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -27759,11 +27767,19 @@
       <c r="E725" s="9" t="n">
         <v>124.99</v>
       </c>
-      <c r="F725" s="8" t="inlineStr"/>
-      <c r="G725" s="8" t="inlineStr"/>
+      <c r="F725" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G725" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H725" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -27789,11 +27805,19 @@
       <c r="E726" s="5" t="n">
         <v>124.99</v>
       </c>
-      <c r="F726" s="4" t="inlineStr"/>
-      <c r="G726" s="4" t="inlineStr"/>
+      <c r="F726" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G726" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H726" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -27819,11 +27843,19 @@
       <c r="E727" s="9" t="n">
         <v>124.99</v>
       </c>
-      <c r="F727" s="8" t="inlineStr"/>
-      <c r="G727" s="8" t="inlineStr"/>
+      <c r="F727" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G727" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H727" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -27849,11 +27881,19 @@
       <c r="E728" s="5" t="n">
         <v>124.99</v>
       </c>
-      <c r="F728" s="4" t="inlineStr"/>
-      <c r="G728" s="4" t="inlineStr"/>
+      <c r="F728" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G728" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H728" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -27879,11 +27919,19 @@
       <c r="E729" s="9" t="n">
         <v>124.99</v>
       </c>
-      <c r="F729" s="8" t="inlineStr"/>
-      <c r="G729" s="8" t="inlineStr"/>
+      <c r="F729" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G729" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H729" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -27909,11 +27957,19 @@
       <c r="E730" s="5" t="n">
         <v>124.99</v>
       </c>
-      <c r="F730" s="4" t="inlineStr"/>
-      <c r="G730" s="4" t="inlineStr"/>
+      <c r="F730" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G730" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H730" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -27939,11 +27995,19 @@
       <c r="E731" s="9" t="n">
         <v>124.99</v>
       </c>
-      <c r="F731" s="8" t="inlineStr"/>
-      <c r="G731" s="8" t="inlineStr"/>
+      <c r="F731" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G731" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H731" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -27969,11 +28033,19 @@
       <c r="E732" s="5" t="n">
         <v>124.99</v>
       </c>
-      <c r="F732" s="4" t="inlineStr"/>
-      <c r="G732" s="4" t="inlineStr"/>
+      <c r="F732" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G732" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H732" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -27999,11 +28071,19 @@
       <c r="E733" s="9" t="n">
         <v>124.99</v>
       </c>
-      <c r="F733" s="8" t="inlineStr"/>
-      <c r="G733" s="8" t="inlineStr"/>
+      <c r="F733" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G733" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H733" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -28029,11 +28109,19 @@
       <c r="E734" s="5" t="n">
         <v>124.99</v>
       </c>
-      <c r="F734" s="4" t="inlineStr"/>
-      <c r="G734" s="4" t="inlineStr"/>
+      <c r="F734" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G734" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H734" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -28059,11 +28147,19 @@
       <c r="E735" s="9" t="n">
         <v>124.99</v>
       </c>
-      <c r="F735" s="8" t="inlineStr"/>
-      <c r="G735" s="8" t="inlineStr"/>
+      <c r="F735" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G735" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H735" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -28199,11 +28295,19 @@
       <c r="E739" s="9" t="n">
         <v>124.99</v>
       </c>
-      <c r="F739" s="8" t="inlineStr"/>
-      <c r="G739" s="8" t="inlineStr"/>
+      <c r="F739" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G739" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H739" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -28297,11 +28401,19 @@
       <c r="E742" s="5" t="n">
         <v>124.99</v>
       </c>
-      <c r="F742" s="4" t="inlineStr"/>
-      <c r="G742" s="4" t="inlineStr"/>
+      <c r="F742" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G742" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H742" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -28327,11 +28439,19 @@
       <c r="E743" s="9" t="n">
         <v>124.99</v>
       </c>
-      <c r="F743" s="8" t="inlineStr"/>
-      <c r="G743" s="8" t="inlineStr"/>
+      <c r="F743" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G743" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H743" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33719,11 +33839,19 @@
       <c r="E905" s="9" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F905" s="8" t="inlineStr"/>
-      <c r="G905" s="8" t="inlineStr"/>
+      <c r="F905" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G905" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H905" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33749,11 +33877,19 @@
       <c r="E906" s="5" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F906" s="4" t="inlineStr"/>
-      <c r="G906" s="4" t="inlineStr"/>
+      <c r="F906" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G906" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H906" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33779,11 +33915,19 @@
       <c r="E907" s="9" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F907" s="8" t="inlineStr"/>
-      <c r="G907" s="8" t="inlineStr"/>
+      <c r="F907" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G907" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H907" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33809,11 +33953,19 @@
       <c r="E908" s="5" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F908" s="4" t="inlineStr"/>
-      <c r="G908" s="4" t="inlineStr"/>
+      <c r="F908" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G908" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H908" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33839,11 +33991,19 @@
       <c r="E909" s="9" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F909" s="8" t="inlineStr"/>
-      <c r="G909" s="8" t="inlineStr"/>
+      <c r="F909" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G909" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H909" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33869,11 +34029,19 @@
       <c r="E910" s="5" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F910" s="4" t="inlineStr"/>
-      <c r="G910" s="4" t="inlineStr"/>
+      <c r="F910" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G910" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H910" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33899,11 +34067,19 @@
       <c r="E911" s="9" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F911" s="8" t="inlineStr"/>
-      <c r="G911" s="8" t="inlineStr"/>
+      <c r="F911" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G911" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H911" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33929,11 +34105,19 @@
       <c r="E912" s="5" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F912" s="4" t="inlineStr"/>
-      <c r="G912" s="4" t="inlineStr"/>
+      <c r="F912" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G912" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H912" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33959,11 +34143,19 @@
       <c r="E913" s="9" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F913" s="8" t="inlineStr"/>
-      <c r="G913" s="8" t="inlineStr"/>
+      <c r="F913" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G913" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H913" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33989,11 +34181,19 @@
       <c r="E914" s="5" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F914" s="4" t="inlineStr"/>
-      <c r="G914" s="4" t="inlineStr"/>
+      <c r="F914" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G914" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H914" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -34019,11 +34219,19 @@
       <c r="E915" s="9" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F915" s="8" t="inlineStr"/>
-      <c r="G915" s="8" t="inlineStr"/>
+      <c r="F915" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G915" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H915" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -34049,11 +34257,19 @@
       <c r="E916" s="5" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F916" s="4" t="inlineStr"/>
-      <c r="G916" s="4" t="inlineStr"/>
+      <c r="F916" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G916" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H916" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -34079,11 +34295,19 @@
       <c r="E917" s="9" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F917" s="8" t="inlineStr"/>
-      <c r="G917" s="8" t="inlineStr"/>
+      <c r="F917" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G917" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H917" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -34109,11 +34333,19 @@
       <c r="E918" s="5" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F918" s="4" t="inlineStr"/>
-      <c r="G918" s="4" t="inlineStr"/>
+      <c r="F918" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G918" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H918" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -34139,11 +34371,19 @@
       <c r="E919" s="9" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F919" s="8" t="inlineStr"/>
-      <c r="G919" s="8" t="inlineStr"/>
+      <c r="F919" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G919" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H919" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -34169,11 +34409,19 @@
       <c r="E920" s="5" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F920" s="4" t="inlineStr"/>
-      <c r="G920" s="4" t="inlineStr"/>
+      <c r="F920" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G920" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H920" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -34199,11 +34447,19 @@
       <c r="E921" s="9" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F921" s="8" t="inlineStr"/>
-      <c r="G921" s="8" t="inlineStr"/>
+      <c r="F921" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G921" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H921" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -34229,11 +34485,19 @@
       <c r="E922" s="5" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F922" s="4" t="inlineStr"/>
-      <c r="G922" s="4" t="inlineStr"/>
+      <c r="F922" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G922" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H922" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -34259,11 +34523,19 @@
       <c r="E923" s="9" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F923" s="8" t="inlineStr"/>
-      <c r="G923" s="8" t="inlineStr"/>
+      <c r="F923" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G923" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H923" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -34289,11 +34561,19 @@
       <c r="E924" s="5" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F924" s="4" t="inlineStr"/>
-      <c r="G924" s="4" t="inlineStr"/>
+      <c r="F924" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G924" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H924" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -35617,11 +35897,19 @@
       <c r="E960" s="5" t="n">
         <v>79.98999999999999</v>
       </c>
-      <c r="F960" s="4" t="inlineStr"/>
-      <c r="G960" s="4" t="inlineStr"/>
+      <c r="F960" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G960" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H960" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -35647,11 +35935,19 @@
       <c r="E961" s="9" t="n">
         <v>79.98999999999999</v>
       </c>
-      <c r="F961" s="8" t="inlineStr"/>
-      <c r="G961" s="8" t="inlineStr"/>
+      <c r="F961" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G961" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H961" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -35677,11 +35973,19 @@
       <c r="E962" s="5" t="n">
         <v>79.98999999999999</v>
       </c>
-      <c r="F962" s="4" t="inlineStr"/>
-      <c r="G962" s="4" t="inlineStr"/>
+      <c r="F962" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G962" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H962" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -35707,11 +36011,19 @@
       <c r="E963" s="9" t="n">
         <v>79.98999999999999</v>
       </c>
-      <c r="F963" s="8" t="inlineStr"/>
-      <c r="G963" s="8" t="inlineStr"/>
+      <c r="F963" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G963" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H963" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -35737,11 +36049,19 @@
       <c r="E964" s="5" t="n">
         <v>69.98999999999999</v>
       </c>
-      <c r="F964" s="4" t="inlineStr"/>
-      <c r="G964" s="4" t="inlineStr"/>
+      <c r="F964" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G964" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H964" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -35767,11 +36087,19 @@
       <c r="E965" s="9" t="n">
         <v>69.98999999999999</v>
       </c>
-      <c r="F965" s="8" t="inlineStr"/>
-      <c r="G965" s="8" t="inlineStr"/>
+      <c r="F965" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G965" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H965" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -35797,11 +36125,19 @@
       <c r="E966" s="5" t="n">
         <v>69.98999999999999</v>
       </c>
-      <c r="F966" s="4" t="inlineStr"/>
-      <c r="G966" s="4" t="inlineStr"/>
+      <c r="F966" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G966" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H966" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -35827,11 +36163,19 @@
       <c r="E967" s="9" t="n">
         <v>69.98999999999999</v>
       </c>
-      <c r="F967" s="8" t="inlineStr"/>
-      <c r="G967" s="8" t="inlineStr"/>
+      <c r="F967" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G967" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H967" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -35857,11 +36201,19 @@
       <c r="E968" s="5" t="n">
         <v>64.98999999999999</v>
       </c>
-      <c r="F968" s="4" t="inlineStr"/>
-      <c r="G968" s="4" t="inlineStr"/>
+      <c r="F968" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G968" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H968" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -35887,11 +36239,19 @@
       <c r="E969" s="9" t="n">
         <v>64.98999999999999</v>
       </c>
-      <c r="F969" s="8" t="inlineStr"/>
-      <c r="G969" s="8" t="inlineStr"/>
+      <c r="F969" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G969" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H969" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -35917,11 +36277,19 @@
       <c r="E970" s="5" t="n">
         <v>64.98999999999999</v>
       </c>
-      <c r="F970" s="4" t="inlineStr"/>
-      <c r="G970" s="4" t="inlineStr"/>
+      <c r="F970" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G970" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H970" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -35947,11 +36315,19 @@
       <c r="E971" s="9" t="n">
         <v>64.98999999999999</v>
       </c>
-      <c r="F971" s="8" t="inlineStr"/>
-      <c r="G971" s="8" t="inlineStr"/>
+      <c r="F971" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G971" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H971" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -35977,11 +36353,19 @@
       <c r="E972" s="5" t="n">
         <v>64.98999999999999</v>
       </c>
-      <c r="F972" s="4" t="inlineStr"/>
-      <c r="G972" s="4" t="inlineStr"/>
+      <c r="F972" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G972" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H972" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -36007,11 +36391,19 @@
       <c r="E973" s="9" t="n">
         <v>64.98999999999999</v>
       </c>
-      <c r="F973" s="8" t="inlineStr"/>
-      <c r="G973" s="8" t="inlineStr"/>
+      <c r="F973" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G973" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H973" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -36037,11 +36429,19 @@
       <c r="E974" s="5" t="n">
         <v>64.98999999999999</v>
       </c>
-      <c r="F974" s="4" t="inlineStr"/>
-      <c r="G974" s="4" t="inlineStr"/>
+      <c r="F974" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G974" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H974" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -36067,11 +36467,19 @@
       <c r="E975" s="9" t="n">
         <v>64.98999999999999</v>
       </c>
-      <c r="F975" s="8" t="inlineStr"/>
-      <c r="G975" s="8" t="inlineStr"/>
+      <c r="F975" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G975" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H975" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -36097,11 +36505,19 @@
       <c r="E976" s="5" t="n">
         <v>64.98999999999999</v>
       </c>
-      <c r="F976" s="4" t="inlineStr"/>
-      <c r="G976" s="4" t="inlineStr"/>
+      <c r="F976" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G976" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H976" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -36127,11 +36543,19 @@
       <c r="E977" s="9" t="n">
         <v>64.98999999999999</v>
       </c>
-      <c r="F977" s="8" t="inlineStr"/>
-      <c r="G977" s="8" t="inlineStr"/>
+      <c r="F977" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G977" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H977" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -36157,11 +36581,19 @@
       <c r="E978" s="5" t="n">
         <v>64.98999999999999</v>
       </c>
-      <c r="F978" s="4" t="inlineStr"/>
-      <c r="G978" s="4" t="inlineStr"/>
+      <c r="F978" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G978" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H978" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -36187,11 +36619,19 @@
       <c r="E979" s="9" t="n">
         <v>64.98999999999999</v>
       </c>
-      <c r="F979" s="8" t="inlineStr"/>
-      <c r="G979" s="8" t="inlineStr"/>
+      <c r="F979" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G979" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H979" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -36217,11 +36657,19 @@
       <c r="E980" s="5" t="n">
         <v>64.98999999999999</v>
       </c>
-      <c r="F980" s="4" t="inlineStr"/>
-      <c r="G980" s="4" t="inlineStr"/>
+      <c r="F980" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G980" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H980" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -36247,11 +36695,19 @@
       <c r="E981" s="9" t="n">
         <v>64.98999999999999</v>
       </c>
-      <c r="F981" s="8" t="inlineStr"/>
-      <c r="G981" s="8" t="inlineStr"/>
+      <c r="F981" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G981" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H981" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -36353,11 +36809,19 @@
       <c r="E984" s="5" t="n">
         <v>61.99</v>
       </c>
-      <c r="F984" s="4" t="inlineStr"/>
-      <c r="G984" s="4" t="inlineStr"/>
+      <c r="F984" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G984" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H984" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -36383,11 +36847,19 @@
       <c r="E985" s="9" t="n">
         <v>61.99</v>
       </c>
-      <c r="F985" s="8" t="inlineStr"/>
-      <c r="G985" s="8" t="inlineStr"/>
+      <c r="F985" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G985" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H985" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -36413,11 +36885,19 @@
       <c r="E986" s="5" t="n">
         <v>61.99</v>
       </c>
-      <c r="F986" s="4" t="inlineStr"/>
-      <c r="G986" s="4" t="inlineStr"/>
+      <c r="F986" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G986" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H986" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -36443,11 +36923,19 @@
       <c r="E987" s="9" t="n">
         <v>61.99</v>
       </c>
-      <c r="F987" s="8" t="inlineStr"/>
-      <c r="G987" s="8" t="inlineStr"/>
+      <c r="F987" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G987" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H987" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -36473,11 +36961,19 @@
       <c r="E988" s="5" t="n">
         <v>61.99</v>
       </c>
-      <c r="F988" s="4" t="inlineStr"/>
-      <c r="G988" s="4" t="inlineStr"/>
+      <c r="F988" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G988" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H988" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -36503,11 +36999,19 @@
       <c r="E989" s="9" t="n">
         <v>61.99</v>
       </c>
-      <c r="F989" s="8" t="inlineStr"/>
-      <c r="G989" s="8" t="inlineStr"/>
+      <c r="F989" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G989" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H989" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -36533,11 +37037,19 @@
       <c r="E990" s="5" t="n">
         <v>61.99</v>
       </c>
-      <c r="F990" s="4" t="inlineStr"/>
-      <c r="G990" s="4" t="inlineStr"/>
+      <c r="F990" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G990" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H990" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -36563,11 +37075,19 @@
       <c r="E991" s="9" t="n">
         <v>61.99</v>
       </c>
-      <c r="F991" s="8" t="inlineStr"/>
-      <c r="G991" s="8" t="inlineStr"/>
+      <c r="F991" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G991" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H991" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -36593,11 +37113,19 @@
       <c r="E992" s="5" t="n">
         <v>61.99</v>
       </c>
-      <c r="F992" s="4" t="inlineStr"/>
-      <c r="G992" s="4" t="inlineStr"/>
+      <c r="F992" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G992" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H992" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -36623,11 +37151,19 @@
       <c r="E993" s="9" t="n">
         <v>61.99</v>
       </c>
-      <c r="F993" s="8" t="inlineStr"/>
-      <c r="G993" s="8" t="inlineStr"/>
+      <c r="F993" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G993" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H993" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -36653,11 +37189,19 @@
       <c r="E994" s="5" t="n">
         <v>61.99</v>
       </c>
-      <c r="F994" s="4" t="inlineStr"/>
-      <c r="G994" s="4" t="inlineStr"/>
+      <c r="F994" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G994" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H994" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -36683,11 +37227,19 @@
       <c r="E995" s="9" t="n">
         <v>61.99</v>
       </c>
-      <c r="F995" s="8" t="inlineStr"/>
-      <c r="G995" s="8" t="inlineStr"/>
+      <c r="F995" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G995" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H995" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -36713,11 +37265,19 @@
       <c r="E996" s="5" t="n">
         <v>61.99</v>
       </c>
-      <c r="F996" s="4" t="inlineStr"/>
-      <c r="G996" s="4" t="inlineStr"/>
+      <c r="F996" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G996" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H996" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -36743,11 +37303,19 @@
       <c r="E997" s="9" t="n">
         <v>61.99</v>
       </c>
-      <c r="F997" s="8" t="inlineStr"/>
-      <c r="G997" s="8" t="inlineStr"/>
+      <c r="F997" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G997" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H997" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -36773,11 +37341,19 @@
       <c r="E998" s="5" t="n">
         <v>61.99</v>
       </c>
-      <c r="F998" s="4" t="inlineStr"/>
-      <c r="G998" s="4" t="inlineStr"/>
+      <c r="F998" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G998" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H998" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -36803,11 +37379,19 @@
       <c r="E999" s="9" t="n">
         <v>61.99</v>
       </c>
-      <c r="F999" s="8" t="inlineStr"/>
-      <c r="G999" s="8" t="inlineStr"/>
+      <c r="F999" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G999" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H999" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -37353,11 +37937,19 @@
       <c r="E1014" s="5" t="n">
         <v>59.99</v>
       </c>
-      <c r="F1014" s="4" t="inlineStr"/>
-      <c r="G1014" s="4" t="inlineStr"/>
+      <c r="F1014" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1014" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1014" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -37383,11 +37975,19 @@
       <c r="E1015" s="9" t="n">
         <v>54.99</v>
       </c>
-      <c r="F1015" s="8" t="inlineStr"/>
-      <c r="G1015" s="8" t="inlineStr"/>
+      <c r="F1015" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1015" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1015" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -41265,7 +41865,7 @@
         </is>
       </c>
       <c r="B27" s="11" t="n">
-        <v>810</v>
+        <v>885</v>
       </c>
     </row>
     <row r="28">
@@ -41275,7 +41875,7 @@
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>239</v>
+        <v>164</v>
       </c>
     </row>
     <row r="29">

</xml_diff>

<commit_message>
Redakcja: 62 nowe karty Piotra i persony do wszystkich
- import 75 dokumentow: 62 nowe karty, 13 nadpisanych nowszymi wersjami
- persony (dla_rodzica + dla_afol) do wszystkich 62 zestawow: sety.json 1010 -> 1072
- poprawki wieku niezgodnego z metryka karty: 77243, 77246 (bylo 18+, przez co
  huby oznaczaly bolidy Speed Champions jako zestawy dla doroslych), 77120, 71052
- rozbieznosci elementow 41758 i 77259 rozstrzygniete Bricksetem na rzecz katalogu
- odswiezone listingi: kolejka, karty poza kolejka, zestawy bez ceny

Kolejka: gotowe 947 (bylo 885), do person 0, do opisania 102.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017crJHR6y9z5CNDcwqQ2UYg
</commit_message>
<xml_diff>
--- a/materialy/kolejka-redakcyjna.xlsx
+++ b/materialy/kolejka-redakcyjna.xlsx
@@ -29837,11 +29837,19 @@
       <c r="E780" s="5" t="n">
         <v>119.99</v>
       </c>
-      <c r="F780" s="4" t="inlineStr"/>
-      <c r="G780" s="4" t="inlineStr"/>
+      <c r="F780" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G780" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H780" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -29867,11 +29875,19 @@
       <c r="E781" s="9" t="n">
         <v>119.99</v>
       </c>
-      <c r="F781" s="8" t="inlineStr"/>
-      <c r="G781" s="8" t="inlineStr"/>
+      <c r="F781" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G781" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H781" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -29897,11 +29913,19 @@
       <c r="E782" s="5" t="n">
         <v>119.99</v>
       </c>
-      <c r="F782" s="4" t="inlineStr"/>
-      <c r="G782" s="4" t="inlineStr"/>
+      <c r="F782" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G782" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H782" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -29927,11 +29951,19 @@
       <c r="E783" s="9" t="n">
         <v>119.99</v>
       </c>
-      <c r="F783" s="8" t="inlineStr"/>
-      <c r="G783" s="8" t="inlineStr"/>
+      <c r="F783" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G783" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H783" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -29957,11 +29989,19 @@
       <c r="E784" s="5" t="n">
         <v>119.99</v>
       </c>
-      <c r="F784" s="4" t="inlineStr"/>
-      <c r="G784" s="4" t="inlineStr"/>
+      <c r="F784" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G784" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H784" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -29987,11 +30027,19 @@
       <c r="E785" s="9" t="n">
         <v>119.99</v>
       </c>
-      <c r="F785" s="8" t="inlineStr"/>
-      <c r="G785" s="8" t="inlineStr"/>
+      <c r="F785" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G785" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H785" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30017,11 +30065,19 @@
       <c r="E786" s="5" t="n">
         <v>119.99</v>
       </c>
-      <c r="F786" s="4" t="inlineStr"/>
-      <c r="G786" s="4" t="inlineStr"/>
+      <c r="F786" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G786" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H786" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30047,11 +30103,19 @@
       <c r="E787" s="9" t="n">
         <v>119.99</v>
       </c>
-      <c r="F787" s="8" t="inlineStr"/>
-      <c r="G787" s="8" t="inlineStr"/>
+      <c r="F787" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G787" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H787" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30077,11 +30141,19 @@
       <c r="E788" s="5" t="n">
         <v>119.99</v>
       </c>
-      <c r="F788" s="4" t="inlineStr"/>
-      <c r="G788" s="4" t="inlineStr"/>
+      <c r="F788" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G788" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H788" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30107,11 +30179,19 @@
       <c r="E789" s="9" t="n">
         <v>119.99</v>
       </c>
-      <c r="F789" s="8" t="inlineStr"/>
-      <c r="G789" s="8" t="inlineStr"/>
+      <c r="F789" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G789" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H789" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30137,11 +30217,19 @@
       <c r="E790" s="5" t="n">
         <v>119.99</v>
       </c>
-      <c r="F790" s="4" t="inlineStr"/>
-      <c r="G790" s="4" t="inlineStr"/>
+      <c r="F790" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G790" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H790" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30167,11 +30255,19 @@
       <c r="E791" s="9" t="n">
         <v>119.99</v>
       </c>
-      <c r="F791" s="8" t="inlineStr"/>
-      <c r="G791" s="8" t="inlineStr"/>
+      <c r="F791" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G791" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H791" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30197,11 +30293,19 @@
       <c r="E792" s="5" t="n">
         <v>119.99</v>
       </c>
-      <c r="F792" s="4" t="inlineStr"/>
-      <c r="G792" s="4" t="inlineStr"/>
+      <c r="F792" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G792" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H792" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30227,11 +30331,19 @@
       <c r="E793" s="9" t="n">
         <v>119.99</v>
       </c>
-      <c r="F793" s="8" t="inlineStr"/>
-      <c r="G793" s="8" t="inlineStr"/>
+      <c r="F793" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G793" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H793" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30257,11 +30369,19 @@
       <c r="E794" s="5" t="n">
         <v>119.99</v>
       </c>
-      <c r="F794" s="4" t="inlineStr"/>
-      <c r="G794" s="4" t="inlineStr"/>
+      <c r="F794" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G794" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H794" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30287,11 +30407,19 @@
       <c r="E795" s="9" t="n">
         <v>119.99</v>
       </c>
-      <c r="F795" s="8" t="inlineStr"/>
-      <c r="G795" s="8" t="inlineStr"/>
+      <c r="F795" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G795" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H795" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30317,11 +30445,19 @@
       <c r="E796" s="5" t="n">
         <v>119.99</v>
       </c>
-      <c r="F796" s="4" t="inlineStr"/>
-      <c r="G796" s="4" t="inlineStr"/>
+      <c r="F796" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G796" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H796" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30347,11 +30483,19 @@
       <c r="E797" s="9" t="n">
         <v>119.99</v>
       </c>
-      <c r="F797" s="8" t="inlineStr"/>
-      <c r="G797" s="8" t="inlineStr"/>
+      <c r="F797" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G797" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H797" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30377,11 +30521,19 @@
       <c r="E798" s="5" t="n">
         <v>114.99</v>
       </c>
-      <c r="F798" s="4" t="inlineStr"/>
-      <c r="G798" s="4" t="inlineStr"/>
+      <c r="F798" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G798" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H798" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30407,11 +30559,19 @@
       <c r="E799" s="9" t="n">
         <v>114.99</v>
       </c>
-      <c r="F799" s="8" t="inlineStr"/>
-      <c r="G799" s="8" t="inlineStr"/>
+      <c r="F799" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G799" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H799" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30437,11 +30597,19 @@
       <c r="E800" s="5" t="n">
         <v>114.99</v>
       </c>
-      <c r="F800" s="4" t="inlineStr"/>
-      <c r="G800" s="4" t="inlineStr"/>
+      <c r="F800" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G800" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H800" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30467,11 +30635,19 @@
       <c r="E801" s="9" t="n">
         <v>114.99</v>
       </c>
-      <c r="F801" s="8" t="inlineStr"/>
-      <c r="G801" s="8" t="inlineStr"/>
+      <c r="F801" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G801" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H801" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30497,11 +30673,19 @@
       <c r="E802" s="5" t="n">
         <v>114.99</v>
       </c>
-      <c r="F802" s="4" t="inlineStr"/>
-      <c r="G802" s="4" t="inlineStr"/>
+      <c r="F802" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G802" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H802" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30527,11 +30711,19 @@
       <c r="E803" s="9" t="n">
         <v>114.99</v>
       </c>
-      <c r="F803" s="8" t="inlineStr"/>
-      <c r="G803" s="8" t="inlineStr"/>
+      <c r="F803" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G803" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H803" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30557,11 +30749,19 @@
       <c r="E804" s="5" t="n">
         <v>114.99</v>
       </c>
-      <c r="F804" s="4" t="inlineStr"/>
-      <c r="G804" s="4" t="inlineStr"/>
+      <c r="F804" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G804" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H804" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30587,11 +30787,19 @@
       <c r="E805" s="9" t="n">
         <v>114.99</v>
       </c>
-      <c r="F805" s="8" t="inlineStr"/>
-      <c r="G805" s="8" t="inlineStr"/>
+      <c r="F805" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G805" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H805" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30617,11 +30825,19 @@
       <c r="E806" s="5" t="n">
         <v>114.99</v>
       </c>
-      <c r="F806" s="4" t="inlineStr"/>
-      <c r="G806" s="4" t="inlineStr"/>
+      <c r="F806" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G806" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H806" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30647,11 +30863,19 @@
       <c r="E807" s="9" t="n">
         <v>114.99</v>
       </c>
-      <c r="F807" s="8" t="inlineStr"/>
-      <c r="G807" s="8" t="inlineStr"/>
+      <c r="F807" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G807" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H807" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30677,11 +30901,19 @@
       <c r="E808" s="5" t="n">
         <v>114.99</v>
       </c>
-      <c r="F808" s="4" t="inlineStr"/>
-      <c r="G808" s="4" t="inlineStr"/>
+      <c r="F808" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G808" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H808" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30707,11 +30939,19 @@
       <c r="E809" s="9" t="n">
         <v>114.99</v>
       </c>
-      <c r="F809" s="8" t="inlineStr"/>
-      <c r="G809" s="8" t="inlineStr"/>
+      <c r="F809" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G809" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H809" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30737,11 +30977,19 @@
       <c r="E810" s="5" t="n">
         <v>114.99</v>
       </c>
-      <c r="F810" s="4" t="inlineStr"/>
-      <c r="G810" s="4" t="inlineStr"/>
+      <c r="F810" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G810" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H810" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30767,11 +31015,19 @@
       <c r="E811" s="9" t="n">
         <v>114.99</v>
       </c>
-      <c r="F811" s="8" t="inlineStr"/>
-      <c r="G811" s="8" t="inlineStr"/>
+      <c r="F811" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G811" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H811" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30797,11 +31053,19 @@
       <c r="E812" s="5" t="n">
         <v>114.99</v>
       </c>
-      <c r="F812" s="4" t="inlineStr"/>
-      <c r="G812" s="4" t="inlineStr"/>
+      <c r="F812" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G812" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H812" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -30827,11 +31091,19 @@
       <c r="E813" s="9" t="n">
         <v>114.99</v>
       </c>
-      <c r="F813" s="8" t="inlineStr"/>
-      <c r="G813" s="8" t="inlineStr"/>
+      <c r="F813" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G813" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H813" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -31389,11 +31661,19 @@
       <c r="E828" s="5" t="n">
         <v>109.99</v>
       </c>
-      <c r="F828" s="4" t="inlineStr"/>
-      <c r="G828" s="4" t="inlineStr"/>
+      <c r="F828" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G828" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H828" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -31419,11 +31699,19 @@
       <c r="E829" s="9" t="n">
         <v>109.99</v>
       </c>
-      <c r="F829" s="8" t="inlineStr"/>
-      <c r="G829" s="8" t="inlineStr"/>
+      <c r="F829" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G829" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H829" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -31449,11 +31737,19 @@
       <c r="E830" s="5" t="n">
         <v>109.99</v>
       </c>
-      <c r="F830" s="4" t="inlineStr"/>
-      <c r="G830" s="4" t="inlineStr"/>
+      <c r="F830" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G830" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H830" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -31479,11 +31775,19 @@
       <c r="E831" s="9" t="n">
         <v>109.99</v>
       </c>
-      <c r="F831" s="8" t="inlineStr"/>
-      <c r="G831" s="8" t="inlineStr"/>
+      <c r="F831" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G831" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H831" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -31509,11 +31813,19 @@
       <c r="E832" s="5" t="n">
         <v>109.99</v>
       </c>
-      <c r="F832" s="4" t="inlineStr"/>
-      <c r="G832" s="4" t="inlineStr"/>
+      <c r="F832" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G832" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H832" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -31539,11 +31851,19 @@
       <c r="E833" s="9" t="n">
         <v>109.99</v>
       </c>
-      <c r="F833" s="8" t="inlineStr"/>
-      <c r="G833" s="8" t="inlineStr"/>
+      <c r="F833" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G833" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H833" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -31569,11 +31889,19 @@
       <c r="E834" s="5" t="n">
         <v>109.99</v>
       </c>
-      <c r="F834" s="4" t="inlineStr"/>
-      <c r="G834" s="4" t="inlineStr"/>
+      <c r="F834" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G834" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H834" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -31599,11 +31927,19 @@
       <c r="E835" s="9" t="n">
         <v>104.99</v>
       </c>
-      <c r="F835" s="8" t="inlineStr"/>
-      <c r="G835" s="8" t="inlineStr"/>
+      <c r="F835" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G835" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H835" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -31629,11 +31965,19 @@
       <c r="E836" s="5" t="n">
         <v>104.99</v>
       </c>
-      <c r="F836" s="4" t="inlineStr"/>
-      <c r="G836" s="4" t="inlineStr"/>
+      <c r="F836" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G836" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H836" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -31659,11 +32003,19 @@
       <c r="E837" s="9" t="n">
         <v>104.99</v>
       </c>
-      <c r="F837" s="8" t="inlineStr"/>
-      <c r="G837" s="8" t="inlineStr"/>
+      <c r="F837" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G837" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H837" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -31689,11 +32041,19 @@
       <c r="E838" s="5" t="n">
         <v>104.99</v>
       </c>
-      <c r="F838" s="4" t="inlineStr"/>
-      <c r="G838" s="4" t="inlineStr"/>
+      <c r="F838" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G838" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H838" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -31719,11 +32079,19 @@
       <c r="E839" s="9" t="n">
         <v>104.99</v>
       </c>
-      <c r="F839" s="8" t="inlineStr"/>
-      <c r="G839" s="8" t="inlineStr"/>
+      <c r="F839" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G839" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H839" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -31859,11 +32227,19 @@
       <c r="E843" s="9" t="n">
         <v>104.99</v>
       </c>
-      <c r="F843" s="8" t="inlineStr"/>
-      <c r="G843" s="8" t="inlineStr"/>
+      <c r="F843" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G843" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H843" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -32307,11 +32683,19 @@
       <c r="E855" s="9" t="n">
         <v>99.98999999999999</v>
       </c>
-      <c r="F855" s="8" t="inlineStr"/>
-      <c r="G855" s="8" t="inlineStr"/>
+      <c r="F855" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G855" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H855" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -32337,11 +32721,19 @@
       <c r="E856" s="5" t="n">
         <v>99.98999999999999</v>
       </c>
-      <c r="F856" s="4" t="inlineStr"/>
-      <c r="G856" s="4" t="inlineStr"/>
+      <c r="F856" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G856" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H856" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -32367,11 +32759,19 @@
       <c r="E857" s="9" t="n">
         <v>99.98999999999999</v>
       </c>
-      <c r="F857" s="8" t="inlineStr"/>
-      <c r="G857" s="8" t="inlineStr"/>
+      <c r="F857" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G857" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H857" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -32397,11 +32797,19 @@
       <c r="E858" s="5" t="n">
         <v>99.98999999999999</v>
       </c>
-      <c r="F858" s="4" t="inlineStr"/>
-      <c r="G858" s="4" t="inlineStr"/>
+      <c r="F858" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G858" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H858" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -32427,11 +32835,19 @@
       <c r="E859" s="9" t="n">
         <v>94.98999999999999</v>
       </c>
-      <c r="F859" s="8" t="inlineStr"/>
-      <c r="G859" s="8" t="inlineStr"/>
+      <c r="F859" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G859" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H859" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -32457,11 +32873,19 @@
       <c r="E860" s="5" t="n">
         <v>89.98999999999999</v>
       </c>
-      <c r="F860" s="4" t="inlineStr"/>
-      <c r="G860" s="4" t="inlineStr"/>
+      <c r="F860" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G860" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H860" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -32487,11 +32911,19 @@
       <c r="E861" s="9" t="n">
         <v>89.98999999999999</v>
       </c>
-      <c r="F861" s="8" t="inlineStr"/>
-      <c r="G861" s="8" t="inlineStr"/>
+      <c r="F861" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G861" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H861" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -32517,11 +32949,19 @@
       <c r="E862" s="5" t="n">
         <v>89.98999999999999</v>
       </c>
-      <c r="F862" s="4" t="inlineStr"/>
-      <c r="G862" s="4" t="inlineStr"/>
+      <c r="F862" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G862" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H862" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -32547,11 +32987,19 @@
       <c r="E863" s="9" t="n">
         <v>89.98999999999999</v>
       </c>
-      <c r="F863" s="8" t="inlineStr"/>
-      <c r="G863" s="8" t="inlineStr"/>
+      <c r="F863" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G863" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H863" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -32577,11 +33025,19 @@
       <c r="E864" s="5" t="n">
         <v>89.98999999999999</v>
       </c>
-      <c r="F864" s="4" t="inlineStr"/>
-      <c r="G864" s="4" t="inlineStr"/>
+      <c r="F864" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G864" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H864" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -32607,11 +33063,19 @@
       <c r="E865" s="9" t="n">
         <v>89.98999999999999</v>
       </c>
-      <c r="F865" s="8" t="inlineStr"/>
-      <c r="G865" s="8" t="inlineStr"/>
+      <c r="F865" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G865" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H865" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -32637,11 +33101,19 @@
       <c r="E866" s="5" t="n">
         <v>89.98999999999999</v>
       </c>
-      <c r="F866" s="4" t="inlineStr"/>
-      <c r="G866" s="4" t="inlineStr"/>
+      <c r="F866" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G866" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H866" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -32667,11 +33139,19 @@
       <c r="E867" s="9" t="n">
         <v>84.98999999999999</v>
       </c>
-      <c r="F867" s="8" t="inlineStr"/>
-      <c r="G867" s="8" t="inlineStr"/>
+      <c r="F867" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G867" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H867" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -32697,11 +33177,19 @@
       <c r="E868" s="5" t="n">
         <v>84.98999999999999</v>
       </c>
-      <c r="F868" s="4" t="inlineStr"/>
-      <c r="G868" s="4" t="inlineStr"/>
+      <c r="F868" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G868" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H868" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -32727,11 +33215,19 @@
       <c r="E869" s="9" t="n">
         <v>84.98999999999999</v>
       </c>
-      <c r="F869" s="8" t="inlineStr"/>
-      <c r="G869" s="8" t="inlineStr"/>
+      <c r="F869" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G869" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H869" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -41865,7 +42361,7 @@
         </is>
       </c>
       <c r="B27" s="11" t="n">
-        <v>885</v>
+        <v>947</v>
       </c>
     </row>
     <row r="28">
@@ -41875,7 +42371,7 @@
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>164</v>
+        <v>102</v>
       </c>
     </row>
     <row r="29">

</xml_diff>

<commit_message>
Redakcja: 95 nowych kart Piotra i persony do wszystkich
- import 156 dokumentow (paczki kolejka 586-617 i braki 001-124): 95 nowych kart
- persony (dla_rodzica + dla_afol) do wszystkich 95: sety.json 1072 -> 1167
- 61 kart przyslanych ponownie bylo identycznych z tymi w repo, nadpisana jedna (40885)
- odswiezone listingi: kolejka, karty poza kolejka, zestawy bez ceny

Kolejka: gotowe 1042 (bylo 947), do person 0, do opisania 7.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017crJHR6y9z5CNDcwqQ2UYg
</commit_message>
<xml_diff>
--- a/materialy/kolejka-redakcyjna.xlsx
+++ b/materialy/kolejka-redakcyjna.xlsx
@@ -33253,11 +33253,19 @@
       <c r="E870" s="5" t="n">
         <v>84.98999999999999</v>
       </c>
-      <c r="F870" s="4" t="inlineStr"/>
-      <c r="G870" s="4" t="inlineStr"/>
+      <c r="F870" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G870" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H870" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33283,11 +33291,19 @@
       <c r="E871" s="9" t="n">
         <v>84.98999999999999</v>
       </c>
-      <c r="F871" s="8" t="inlineStr"/>
-      <c r="G871" s="8" t="inlineStr"/>
+      <c r="F871" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G871" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H871" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33313,11 +33329,19 @@
       <c r="E872" s="5" t="n">
         <v>84.98999999999999</v>
       </c>
-      <c r="F872" s="4" t="inlineStr"/>
-      <c r="G872" s="4" t="inlineStr"/>
+      <c r="F872" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G872" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H872" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33343,11 +33367,19 @@
       <c r="E873" s="9" t="n">
         <v>84.98999999999999</v>
       </c>
-      <c r="F873" s="8" t="inlineStr"/>
-      <c r="G873" s="8" t="inlineStr"/>
+      <c r="F873" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G873" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H873" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33373,11 +33405,19 @@
       <c r="E874" s="5" t="n">
         <v>84.98999999999999</v>
       </c>
-      <c r="F874" s="4" t="inlineStr"/>
-      <c r="G874" s="4" t="inlineStr"/>
+      <c r="F874" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G874" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H874" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33403,11 +33443,19 @@
       <c r="E875" s="9" t="n">
         <v>84.98999999999999</v>
       </c>
-      <c r="F875" s="8" t="inlineStr"/>
-      <c r="G875" s="8" t="inlineStr"/>
+      <c r="F875" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G875" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H875" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33433,11 +33481,19 @@
       <c r="E876" s="5" t="n">
         <v>84.98999999999999</v>
       </c>
-      <c r="F876" s="4" t="inlineStr"/>
-      <c r="G876" s="4" t="inlineStr"/>
+      <c r="F876" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G876" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H876" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33463,11 +33519,19 @@
       <c r="E877" s="9" t="n">
         <v>84.98999999999999</v>
       </c>
-      <c r="F877" s="8" t="inlineStr"/>
-      <c r="G877" s="8" t="inlineStr"/>
+      <c r="F877" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G877" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H877" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33493,11 +33557,19 @@
       <c r="E878" s="5" t="n">
         <v>84.98999999999999</v>
       </c>
-      <c r="F878" s="4" t="inlineStr"/>
-      <c r="G878" s="4" t="inlineStr"/>
+      <c r="F878" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G878" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H878" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33523,11 +33595,19 @@
       <c r="E879" s="9" t="n">
         <v>84.98999999999999</v>
       </c>
-      <c r="F879" s="8" t="inlineStr"/>
-      <c r="G879" s="8" t="inlineStr"/>
+      <c r="F879" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G879" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H879" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33553,11 +33633,19 @@
       <c r="E880" s="5" t="n">
         <v>84.98999999999999</v>
       </c>
-      <c r="F880" s="4" t="inlineStr"/>
-      <c r="G880" s="4" t="inlineStr"/>
+      <c r="F880" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G880" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H880" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33583,11 +33671,19 @@
       <c r="E881" s="9" t="n">
         <v>84.98999999999999</v>
       </c>
-      <c r="F881" s="8" t="inlineStr"/>
-      <c r="G881" s="8" t="inlineStr"/>
+      <c r="F881" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G881" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H881" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33613,11 +33709,19 @@
       <c r="E882" s="5" t="n">
         <v>84.98999999999999</v>
       </c>
-      <c r="F882" s="4" t="inlineStr"/>
-      <c r="G882" s="4" t="inlineStr"/>
+      <c r="F882" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G882" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H882" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33643,11 +33747,19 @@
       <c r="E883" s="9" t="n">
         <v>84.98999999999999</v>
       </c>
-      <c r="F883" s="8" t="inlineStr"/>
-      <c r="G883" s="8" t="inlineStr"/>
+      <c r="F883" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G883" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H883" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33673,11 +33785,19 @@
       <c r="E884" s="5" t="n">
         <v>84.98999999999999</v>
       </c>
-      <c r="F884" s="4" t="inlineStr"/>
-      <c r="G884" s="4" t="inlineStr"/>
+      <c r="F884" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G884" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H884" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33703,11 +33823,19 @@
       <c r="E885" s="9" t="n">
         <v>84.98999999999999</v>
       </c>
-      <c r="F885" s="8" t="inlineStr"/>
-      <c r="G885" s="8" t="inlineStr"/>
+      <c r="F885" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G885" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H885" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33733,11 +33861,19 @@
       <c r="E886" s="5" t="n">
         <v>84.98999999999999</v>
       </c>
-      <c r="F886" s="4" t="inlineStr"/>
-      <c r="G886" s="4" t="inlineStr"/>
+      <c r="F886" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G886" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H886" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33763,11 +33899,19 @@
       <c r="E887" s="9" t="n">
         <v>84.98999999999999</v>
       </c>
-      <c r="F887" s="8" t="inlineStr"/>
-      <c r="G887" s="8" t="inlineStr"/>
+      <c r="F887" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G887" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H887" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33945,11 +34089,19 @@
       <c r="E892" s="5" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F892" s="4" t="inlineStr"/>
-      <c r="G892" s="4" t="inlineStr"/>
+      <c r="F892" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G892" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H892" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -33975,11 +34127,19 @@
       <c r="E893" s="9" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F893" s="8" t="inlineStr"/>
-      <c r="G893" s="8" t="inlineStr"/>
+      <c r="F893" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G893" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H893" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -34005,11 +34165,19 @@
       <c r="E894" s="5" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F894" s="4" t="inlineStr"/>
-      <c r="G894" s="4" t="inlineStr"/>
+      <c r="F894" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G894" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H894" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -34035,11 +34203,19 @@
       <c r="E895" s="9" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F895" s="8" t="inlineStr"/>
-      <c r="G895" s="8" t="inlineStr"/>
+      <c r="F895" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G895" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H895" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -34065,11 +34241,19 @@
       <c r="E896" s="5" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F896" s="4" t="inlineStr"/>
-      <c r="G896" s="4" t="inlineStr"/>
+      <c r="F896" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G896" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H896" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -34095,11 +34279,19 @@
       <c r="E897" s="9" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F897" s="8" t="inlineStr"/>
-      <c r="G897" s="8" t="inlineStr"/>
+      <c r="F897" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G897" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H897" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -34125,11 +34317,19 @@
       <c r="E898" s="5" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F898" s="4" t="inlineStr"/>
-      <c r="G898" s="4" t="inlineStr"/>
+      <c r="F898" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G898" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H898" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -34155,11 +34355,19 @@
       <c r="E899" s="9" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F899" s="8" t="inlineStr"/>
-      <c r="G899" s="8" t="inlineStr"/>
+      <c r="F899" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G899" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H899" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -34185,11 +34393,19 @@
       <c r="E900" s="5" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F900" s="4" t="inlineStr"/>
-      <c r="G900" s="4" t="inlineStr"/>
+      <c r="F900" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G900" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H900" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -34215,11 +34431,19 @@
       <c r="E901" s="9" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F901" s="8" t="inlineStr"/>
-      <c r="G901" s="8" t="inlineStr"/>
+      <c r="F901" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G901" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H901" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -34245,11 +34469,19 @@
       <c r="E902" s="5" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F902" s="4" t="inlineStr"/>
-      <c r="G902" s="4" t="inlineStr"/>
+      <c r="F902" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G902" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H902" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -34275,11 +34507,19 @@
       <c r="E903" s="9" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F903" s="8" t="inlineStr"/>
-      <c r="G903" s="8" t="inlineStr"/>
+      <c r="F903" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G903" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H903" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -34305,11 +34545,19 @@
       <c r="E904" s="5" t="n">
         <v>81.98999999999999</v>
       </c>
-      <c r="F904" s="4" t="inlineStr"/>
-      <c r="G904" s="4" t="inlineStr"/>
+      <c r="F904" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G904" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H904" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -38509,11 +38757,19 @@
       <c r="E1016" s="5" t="n">
         <v>54.99</v>
       </c>
-      <c r="F1016" s="4" t="inlineStr"/>
-      <c r="G1016" s="4" t="inlineStr"/>
+      <c r="F1016" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1016" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1016" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -38539,11 +38795,19 @@
       <c r="E1017" s="9" t="n">
         <v>54.99</v>
       </c>
-      <c r="F1017" s="8" t="inlineStr"/>
-      <c r="G1017" s="8" t="inlineStr"/>
+      <c r="F1017" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1017" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1017" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -38569,11 +38833,19 @@
       <c r="E1018" s="5" t="n">
         <v>54.99</v>
       </c>
-      <c r="F1018" s="4" t="inlineStr"/>
-      <c r="G1018" s="4" t="inlineStr"/>
+      <c r="F1018" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1018" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1018" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -38599,11 +38871,19 @@
       <c r="E1019" s="9" t="n">
         <v>54.99</v>
       </c>
-      <c r="F1019" s="8" t="inlineStr"/>
-      <c r="G1019" s="8" t="inlineStr"/>
+      <c r="F1019" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1019" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1019" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -38629,11 +38909,19 @@
       <c r="E1020" s="5" t="n">
         <v>54.99</v>
       </c>
-      <c r="F1020" s="4" t="inlineStr"/>
-      <c r="G1020" s="4" t="inlineStr"/>
+      <c r="F1020" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1020" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1020" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -38659,11 +38947,19 @@
       <c r="E1021" s="9" t="n">
         <v>54.99</v>
       </c>
-      <c r="F1021" s="8" t="inlineStr"/>
-      <c r="G1021" s="8" t="inlineStr"/>
+      <c r="F1021" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1021" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1021" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -38689,11 +38985,19 @@
       <c r="E1022" s="5" t="n">
         <v>54.99</v>
       </c>
-      <c r="F1022" s="4" t="inlineStr"/>
-      <c r="G1022" s="4" t="inlineStr"/>
+      <c r="F1022" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1022" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1022" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -38719,11 +39023,19 @@
       <c r="E1023" s="9" t="n">
         <v>54.99</v>
       </c>
-      <c r="F1023" s="8" t="inlineStr"/>
-      <c r="G1023" s="8" t="inlineStr"/>
+      <c r="F1023" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1023" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1023" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -38787,11 +39099,19 @@
       <c r="E1025" s="9" t="n">
         <v>45.99</v>
       </c>
-      <c r="F1025" s="8" t="inlineStr"/>
-      <c r="G1025" s="8" t="inlineStr"/>
+      <c r="F1025" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1025" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1025" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -38817,11 +39137,19 @@
       <c r="E1026" s="5" t="n">
         <v>45.99</v>
       </c>
-      <c r="F1026" s="4" t="inlineStr"/>
-      <c r="G1026" s="4" t="inlineStr"/>
+      <c r="F1026" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1026" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1026" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -38847,11 +39175,19 @@
       <c r="E1027" s="9" t="n">
         <v>42.99</v>
       </c>
-      <c r="F1027" s="8" t="inlineStr"/>
-      <c r="G1027" s="8" t="inlineStr"/>
+      <c r="F1027" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1027" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1027" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -38877,11 +39213,19 @@
       <c r="E1028" s="5" t="n">
         <v>42.99</v>
       </c>
-      <c r="F1028" s="4" t="inlineStr"/>
-      <c r="G1028" s="4" t="inlineStr"/>
+      <c r="F1028" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1028" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1028" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -38907,11 +39251,19 @@
       <c r="E1029" s="9" t="n">
         <v>42.99</v>
       </c>
-      <c r="F1029" s="8" t="inlineStr"/>
-      <c r="G1029" s="8" t="inlineStr"/>
+      <c r="F1029" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1029" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1029" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -38937,11 +39289,19 @@
       <c r="E1030" s="5" t="n">
         <v>42.99</v>
       </c>
-      <c r="F1030" s="4" t="inlineStr"/>
-      <c r="G1030" s="4" t="inlineStr"/>
+      <c r="F1030" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1030" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1030" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -38967,11 +39327,19 @@
       <c r="E1031" s="9" t="n">
         <v>42.99</v>
       </c>
-      <c r="F1031" s="8" t="inlineStr"/>
-      <c r="G1031" s="8" t="inlineStr"/>
+      <c r="F1031" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1031" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1031" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -38997,11 +39365,19 @@
       <c r="E1032" s="5" t="n">
         <v>42.99</v>
       </c>
-      <c r="F1032" s="4" t="inlineStr"/>
-      <c r="G1032" s="4" t="inlineStr"/>
+      <c r="F1032" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1032" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1032" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -39027,11 +39403,19 @@
       <c r="E1033" s="9" t="n">
         <v>42.99</v>
       </c>
-      <c r="F1033" s="8" t="inlineStr"/>
-      <c r="G1033" s="8" t="inlineStr"/>
+      <c r="F1033" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1033" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1033" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -39057,11 +39441,19 @@
       <c r="E1034" s="5" t="n">
         <v>42.99</v>
       </c>
-      <c r="F1034" s="4" t="inlineStr"/>
-      <c r="G1034" s="4" t="inlineStr"/>
+      <c r="F1034" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1034" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1034" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -39087,11 +39479,19 @@
       <c r="E1035" s="9" t="n">
         <v>42.99</v>
       </c>
-      <c r="F1035" s="8" t="inlineStr"/>
-      <c r="G1035" s="8" t="inlineStr"/>
+      <c r="F1035" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1035" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1035" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -39117,11 +39517,19 @@
       <c r="E1036" s="5" t="n">
         <v>42.99</v>
       </c>
-      <c r="F1036" s="4" t="inlineStr"/>
-      <c r="G1036" s="4" t="inlineStr"/>
+      <c r="F1036" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1036" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1036" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -39147,11 +39555,19 @@
       <c r="E1037" s="9" t="n">
         <v>42.99</v>
       </c>
-      <c r="F1037" s="8" t="inlineStr"/>
-      <c r="G1037" s="8" t="inlineStr"/>
+      <c r="F1037" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1037" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1037" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -39177,11 +39593,19 @@
       <c r="E1038" s="5" t="n">
         <v>42.99</v>
       </c>
-      <c r="F1038" s="4" t="inlineStr"/>
-      <c r="G1038" s="4" t="inlineStr"/>
+      <c r="F1038" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1038" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1038" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -39207,11 +39631,19 @@
       <c r="E1039" s="9" t="n">
         <v>42.99</v>
       </c>
-      <c r="F1039" s="8" t="inlineStr"/>
-      <c r="G1039" s="8" t="inlineStr"/>
+      <c r="F1039" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1039" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1039" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -39237,11 +39669,19 @@
       <c r="E1040" s="5" t="n">
         <v>42.99</v>
       </c>
-      <c r="F1040" s="4" t="inlineStr"/>
-      <c r="G1040" s="4" t="inlineStr"/>
+      <c r="F1040" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1040" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1040" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -39267,11 +39707,19 @@
       <c r="E1041" s="9" t="n">
         <v>42.99</v>
       </c>
-      <c r="F1041" s="8" t="inlineStr"/>
-      <c r="G1041" s="8" t="inlineStr"/>
+      <c r="F1041" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1041" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1041" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -39297,11 +39745,19 @@
       <c r="E1042" s="5" t="n">
         <v>41.99</v>
       </c>
-      <c r="F1042" s="4" t="inlineStr"/>
-      <c r="G1042" s="4" t="inlineStr"/>
+      <c r="F1042" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1042" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1042" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -39327,11 +39783,19 @@
       <c r="E1043" s="9" t="n">
         <v>41.99</v>
       </c>
-      <c r="F1043" s="8" t="inlineStr"/>
-      <c r="G1043" s="8" t="inlineStr"/>
+      <c r="F1043" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1043" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1043" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -39357,11 +39821,19 @@
       <c r="E1044" s="5" t="n">
         <v>41.99</v>
       </c>
-      <c r="F1044" s="4" t="inlineStr"/>
-      <c r="G1044" s="4" t="inlineStr"/>
+      <c r="F1044" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1044" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1044" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -39387,11 +39859,19 @@
       <c r="E1045" s="9" t="n">
         <v>41.99</v>
       </c>
-      <c r="F1045" s="8" t="inlineStr"/>
-      <c r="G1045" s="8" t="inlineStr"/>
+      <c r="F1045" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1045" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1045" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -39417,11 +39897,19 @@
       <c r="E1046" s="5" t="n">
         <v>41.99</v>
       </c>
-      <c r="F1046" s="4" t="inlineStr"/>
-      <c r="G1046" s="4" t="inlineStr"/>
+      <c r="F1046" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1046" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1046" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -39447,11 +39935,19 @@
       <c r="E1047" s="9" t="n">
         <v>41.99</v>
       </c>
-      <c r="F1047" s="8" t="inlineStr"/>
-      <c r="G1047" s="8" t="inlineStr"/>
+      <c r="F1047" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1047" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1047" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -39477,11 +39973,19 @@
       <c r="E1048" s="5" t="n">
         <v>41.99</v>
       </c>
-      <c r="F1048" s="4" t="inlineStr"/>
-      <c r="G1048" s="4" t="inlineStr"/>
+      <c r="F1048" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1048" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1048" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -39507,11 +40011,19 @@
       <c r="E1049" s="9" t="n">
         <v>41.99</v>
       </c>
-      <c r="F1049" s="8" t="inlineStr"/>
-      <c r="G1049" s="8" t="inlineStr"/>
+      <c r="F1049" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1049" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1049" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -39537,11 +40049,19 @@
       <c r="E1050" s="5" t="n">
         <v>41.99</v>
       </c>
-      <c r="F1050" s="4" t="inlineStr"/>
-      <c r="G1050" s="4" t="inlineStr"/>
+      <c r="F1050" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1050" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1050" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -39567,11 +40087,19 @@
       <c r="E1051" s="9" t="n">
         <v>41.99</v>
       </c>
-      <c r="F1051" s="8" t="inlineStr"/>
-      <c r="G1051" s="8" t="inlineStr"/>
+      <c r="F1051" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1051" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1051" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -39597,11 +40125,19 @@
       <c r="E1052" s="5" t="n">
         <v>41.99</v>
       </c>
-      <c r="F1052" s="4" t="inlineStr"/>
-      <c r="G1052" s="4" t="inlineStr"/>
+      <c r="F1052" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1052" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1052" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -39627,11 +40163,19 @@
       <c r="E1053" s="9" t="n">
         <v>41.99</v>
       </c>
-      <c r="F1053" s="8" t="inlineStr"/>
-      <c r="G1053" s="8" t="inlineStr"/>
+      <c r="F1053" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1053" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1053" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -39657,11 +40201,19 @@
       <c r="E1054" s="5" t="n">
         <v>41.99</v>
       </c>
-      <c r="F1054" s="4" t="inlineStr"/>
-      <c r="G1054" s="4" t="inlineStr"/>
+      <c r="F1054" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1054" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1054" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -40689,11 +41241,19 @@
       <c r="E1082" s="5" t="n">
         <v>39.99</v>
       </c>
-      <c r="F1082" s="4" t="inlineStr"/>
-      <c r="G1082" s="4" t="inlineStr"/>
+      <c r="F1082" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1082" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1082" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -40719,11 +41279,19 @@
       <c r="E1083" s="9" t="n">
         <v>39.99</v>
       </c>
-      <c r="F1083" s="8" t="inlineStr"/>
-      <c r="G1083" s="8" t="inlineStr"/>
+      <c r="F1083" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1083" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1083" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -40749,11 +41317,19 @@
       <c r="E1084" s="5" t="n">
         <v>39.99</v>
       </c>
-      <c r="F1084" s="4" t="inlineStr"/>
-      <c r="G1084" s="4" t="inlineStr"/>
+      <c r="F1084" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1084" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1084" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -40779,11 +41355,19 @@
       <c r="E1085" s="9" t="n">
         <v>36.99</v>
       </c>
-      <c r="F1085" s="8" t="inlineStr"/>
-      <c r="G1085" s="8" t="inlineStr"/>
+      <c r="F1085" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1085" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1085" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -40809,11 +41393,19 @@
       <c r="E1086" s="5" t="n">
         <v>36.99</v>
       </c>
-      <c r="F1086" s="4" t="inlineStr"/>
-      <c r="G1086" s="4" t="inlineStr"/>
+      <c r="F1086" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1086" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1086" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -40839,11 +41431,19 @@
       <c r="E1087" s="9" t="n">
         <v>36.99</v>
       </c>
-      <c r="F1087" s="8" t="inlineStr"/>
-      <c r="G1087" s="8" t="inlineStr"/>
+      <c r="F1087" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1087" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1087" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -40907,11 +41507,19 @@
       <c r="E1089" s="9" t="n">
         <v>17.99</v>
       </c>
-      <c r="F1089" s="8" t="inlineStr"/>
-      <c r="G1089" s="8" t="inlineStr"/>
+      <c r="F1089" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1089" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1089" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -40937,11 +41545,19 @@
       <c r="E1090" s="5" t="n">
         <v>17.99</v>
       </c>
-      <c r="F1090" s="4" t="inlineStr"/>
-      <c r="G1090" s="4" t="inlineStr"/>
+      <c r="F1090" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1090" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1090" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -40967,11 +41583,19 @@
       <c r="E1091" s="9" t="n">
         <v>16.99</v>
       </c>
-      <c r="F1091" s="8" t="inlineStr"/>
-      <c r="G1091" s="8" t="inlineStr"/>
+      <c r="F1091" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1091" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1091" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -40997,11 +41621,19 @@
       <c r="E1092" s="5" t="n">
         <v>16.99</v>
       </c>
-      <c r="F1092" s="4" t="inlineStr"/>
-      <c r="G1092" s="4" t="inlineStr"/>
+      <c r="F1092" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1092" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1092" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -41027,11 +41659,19 @@
       <c r="E1093" s="9" t="n">
         <v>16.99</v>
       </c>
-      <c r="F1093" s="8" t="inlineStr"/>
-      <c r="G1093" s="8" t="inlineStr"/>
+      <c r="F1093" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1093" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1093" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -41057,11 +41697,19 @@
       <c r="E1094" s="5" t="n">
         <v>16.99</v>
       </c>
-      <c r="F1094" s="4" t="inlineStr"/>
-      <c r="G1094" s="4" t="inlineStr"/>
+      <c r="F1094" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1094" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1094" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -41087,11 +41735,19 @@
       <c r="E1095" s="9" t="n">
         <v>16.99</v>
       </c>
-      <c r="F1095" s="8" t="inlineStr"/>
-      <c r="G1095" s="8" t="inlineStr"/>
+      <c r="F1095" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1095" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1095" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -41117,11 +41773,19 @@
       <c r="E1096" s="5" t="n">
         <v>16.99</v>
       </c>
-      <c r="F1096" s="4" t="inlineStr"/>
-      <c r="G1096" s="4" t="inlineStr"/>
+      <c r="F1096" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1096" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1096" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -41147,11 +41811,19 @@
       <c r="E1097" s="9" t="n">
         <v>16.99</v>
       </c>
-      <c r="F1097" s="8" t="inlineStr"/>
-      <c r="G1097" s="8" t="inlineStr"/>
+      <c r="F1097" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1097" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1097" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -41177,11 +41849,19 @@
       <c r="E1098" s="5" t="n">
         <v>16.99</v>
       </c>
-      <c r="F1098" s="4" t="inlineStr"/>
-      <c r="G1098" s="4" t="inlineStr"/>
+      <c r="F1098" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1098" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1098" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -41207,11 +41887,19 @@
       <c r="E1099" s="9" t="n">
         <v>16.99</v>
       </c>
-      <c r="F1099" s="8" t="inlineStr"/>
-      <c r="G1099" s="8" t="inlineStr"/>
+      <c r="F1099" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1099" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1099" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -41237,11 +41925,19 @@
       <c r="E1100" s="5" t="n">
         <v>16.99</v>
       </c>
-      <c r="F1100" s="4" t="inlineStr"/>
-      <c r="G1100" s="4" t="inlineStr"/>
+      <c r="F1100" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1100" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1100" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -41267,11 +41963,19 @@
       <c r="E1101" s="9" t="n">
         <v>16.99</v>
       </c>
-      <c r="F1101" s="8" t="inlineStr"/>
-      <c r="G1101" s="8" t="inlineStr"/>
+      <c r="F1101" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1101" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1101" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -41297,11 +42001,19 @@
       <c r="E1102" s="5" t="n">
         <v>16.99</v>
       </c>
-      <c r="F1102" s="4" t="inlineStr"/>
-      <c r="G1102" s="4" t="inlineStr"/>
+      <c r="F1102" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1102" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1102" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -41327,11 +42039,19 @@
       <c r="E1103" s="9" t="n">
         <v>16.99</v>
       </c>
-      <c r="F1103" s="8" t="inlineStr"/>
-      <c r="G1103" s="8" t="inlineStr"/>
+      <c r="F1103" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1103" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1103" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -41357,11 +42077,19 @@
       <c r="E1104" s="5" t="n">
         <v>16.99</v>
       </c>
-      <c r="F1104" s="4" t="inlineStr"/>
-      <c r="G1104" s="4" t="inlineStr"/>
+      <c r="F1104" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1104" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1104" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -41387,11 +42115,19 @@
       <c r="E1105" s="9" t="n">
         <v>16.99</v>
       </c>
-      <c r="F1105" s="8" t="inlineStr"/>
-      <c r="G1105" s="8" t="inlineStr"/>
+      <c r="F1105" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1105" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1105" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -41417,11 +42153,19 @@
       <c r="E1106" s="5" t="n">
         <v>16.99</v>
       </c>
-      <c r="F1106" s="4" t="inlineStr"/>
-      <c r="G1106" s="4" t="inlineStr"/>
+      <c r="F1106" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1106" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1106" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -41447,11 +42191,19 @@
       <c r="E1107" s="9" t="n">
         <v>16.99</v>
       </c>
-      <c r="F1107" s="8" t="inlineStr"/>
-      <c r="G1107" s="8" t="inlineStr"/>
+      <c r="F1107" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1107" s="8" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1107" s="7" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -42085,11 +42837,19 @@
       <c r="E1124" s="5" t="n">
         <v>14.99</v>
       </c>
-      <c r="F1124" s="4" t="inlineStr"/>
-      <c r="G1124" s="4" t="inlineStr"/>
+      <c r="F1124" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="G1124" s="4" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H1124" s="3" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>gotowe</t>
         </is>
       </c>
     </row>
@@ -42361,27 +43121,27 @@
         </is>
       </c>
       <c r="B27" s="11" t="n">
-        <v>947</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t>do opisania</t>
+          <t>nasz opis - czeka na karte</t>
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>102</v>
+        <v>74</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t>nasz opis - czeka na karte</t>
+          <t>do opisania</t>
         </is>
       </c>
       <c r="B29" s="11" t="n">
-        <v>74</v>
+        <v>7</v>
       </c>
     </row>
     <row r="30">

</xml_diff>